<commit_message>
Paso 2: núcleo de reglas y simulación T1-T12
</commit_message>
<xml_diff>
--- a/planilla/contenido_alfa.xlsx
+++ b/planilla/contenido_alfa.xlsx
@@ -11,24 +11,25 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="objetos" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="salas" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="guion" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="textos" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="anotaciones" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="items" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="audios" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="eventos" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="config" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="conexiones" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="textos" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="anotaciones" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="items" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="audios" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="eventos" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="config" sheetId="11" state="visible" r:id="rId11"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'LEEME'!$A$1:$A$17</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'objetos'!$A$1:$X$55</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'salas'!$A$1:$I$5</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'guion'!$A$1:$E$13</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'textos'!$A$1:$D$68</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'anotaciones'!$A$1:$B$21</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'items'!$A$1:$C$2</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'audios'!$A$1:$B$3</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'eventos'!$A$1:$B$3</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'config'!$A$1:$C$7</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'textos'!$A$1:$D$68</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'anotaciones'!$A$1:$B$21</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'items'!$A$1:$C$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'audios'!$A$1:$B$3</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'eventos'!$A$1:$B$3</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'config'!$A$1:$C$7</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -80,7 +81,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
@@ -88,6 +89,8 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -453,7 +456,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A17"/>
+  <dimension ref="A1:A18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="140" customWidth="1" min="1" max="1"/>
@@ -567,6 +570,13 @@
       <c r="A17" s="2" t="inlineStr">
         <is>
           <t>Los textos son BORRADORES (el texto final se escribe en el paso 9). Regla anti-spoiler: ver diseno/05, sección 0.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="3" t="inlineStr">
+        <is>
+          <t>Conexiones: cada fila es una conexión de ida y vuelta entre dos salas.</t>
         </is>
       </c>
     </row>
@@ -582,7 +592,62 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C7"/>
+  <dimension ref="A1:B3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="80" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>descripcion</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>arreglo_com</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Comunicaciones pasa a poder tener luz máxima (3).</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>desbloquear_SCO</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Desbloquea la sala común. Queda con luz 0.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:B3"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -694,6 +759,21 @@
       <c r="C7" s="2" t="inlineStr">
         <is>
           <t>Cantidad de turnos del Alfa</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>costo_volver_a_mando</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>Moverse a la sala de mando no cuesta energía (01, sección 4)</t>
         </is>
       </c>
     </row>
@@ -5380,6 +5460,93 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:C4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="60" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>desde</t>
+        </is>
+      </c>
+      <c r="B1" s="4" t="inlineStr">
+        <is>
+          <t>hasta</t>
+        </is>
+      </c>
+      <c r="C1" s="4" t="inlineStr">
+        <is>
+          <t>notas</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>MAN</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>COM</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>Pasillo corto (1 ↔ 2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>COM</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>PTA</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Pasillo corto hacia arriba (2 ↔ 4)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>COM</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>SCO</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>Puerta bloqueada al inicio: se abre con COM_Q (2 ↔ 3)</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:D68"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -6757,7 +6924,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -7028,7 +7195,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -7082,7 +7249,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -7135,59 +7302,4 @@
   <autoFilter ref="A1:B3"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:B3"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="18" customWidth="1" min="1" max="1"/>
-    <col width="80" customWidth="1" min="2" max="2"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>id</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>descripcion</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>arreglo_com</t>
-        </is>
-      </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>Comunicaciones pasa a poder tener luz máxima (3).</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>desbloquear_SCO</t>
-        </is>
-      </c>
-      <c r="B3" s="2" t="inlineStr">
-        <is>
-          <t>Desbloquea la sala común. Queda con luz 0.</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <autoFilter ref="A1:B3"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
Paso 4: objetos, interacción, zoom y menú de pausa
</commit_message>
<xml_diff>
--- a/planilla/contenido_alfa.xlsx
+++ b/planilla/contenido_alfa.xlsx
@@ -21,7 +21,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'LEEME'!$A$1:$A$17</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'objetos'!$A$1:$X$55</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'objetos'!$A$1:$AB$55</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'salas'!$A$1:$I$5</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'guion'!$A$1:$E$13</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'textos'!$A$1:$D$68</definedName>
@@ -456,7 +456,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A18"/>
+  <dimension ref="A1:A19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="140" customWidth="1" min="1" max="1"/>
@@ -577,6 +577,13 @@
       <c r="A18" s="3" t="inlineStr">
         <is>
           <t>Conexiones: cada fila es una conexión de ida y vuelta entre dos salas.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="3" t="inlineStr">
+        <is>
+          <t>Posición de cada objeto: x, y, ancho, alto en tiles de 16 px, desde la esquina de arriba a la izquierda de la sala (la pared ocupa medio tile). Las conversaciones de NORA comparten el lugar de la consola.</t>
         </is>
       </c>
     </row>
@@ -789,7 +796,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X55"/>
+  <dimension ref="A1:AB55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -816,6 +823,10 @@
     <col width="6" customWidth="1" min="22" max="22"/>
     <col width="16" customWidth="1" min="23" max="23"/>
     <col width="40" customWidth="1" min="24" max="24"/>
+    <col width="6" customWidth="1" min="25" max="25"/>
+    <col width="6" customWidth="1" min="26" max="26"/>
+    <col width="6" customWidth="1" min="27" max="27"/>
+    <col width="6" customWidth="1" min="28" max="28"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -939,6 +950,26 @@
           <t>notas</t>
         </is>
       </c>
+      <c r="Y1" s="4" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="Z1" s="4" t="inlineStr">
+        <is>
+          <t>y</t>
+        </is>
+      </c>
+      <c r="AA1" s="4" t="inlineStr">
+        <is>
+          <t>ancho</t>
+        </is>
+      </c>
+      <c r="AB1" s="4" t="inlineStr">
+        <is>
+          <t>alto</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -1025,6 +1056,18 @@
       <c r="V2" s="2" t="n"/>
       <c r="W2" s="2" t="n"/>
       <c r="X2" s="2" t="inlineStr"/>
+      <c r="Y2" s="3" t="n">
+        <v>9</v>
+      </c>
+      <c r="Z2" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="AA2" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="AB2" s="3" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -1091,6 +1134,18 @@
       <c r="V3" s="2" t="n"/>
       <c r="W3" s="2" t="n"/>
       <c r="X3" s="2" t="inlineStr"/>
+      <c r="Y3" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="Z3" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="AA3" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="AB3" s="3" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -1157,6 +1212,18 @@
       <c r="V4" s="2" t="n"/>
       <c r="W4" s="2" t="n"/>
       <c r="X4" s="2" t="inlineStr"/>
+      <c r="Y4" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="Z4" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="AA4" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="AB4" s="3" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -1223,6 +1290,18 @@
       <c r="V5" s="2" t="n"/>
       <c r="W5" s="2" t="n"/>
       <c r="X5" s="2" t="inlineStr"/>
+      <c r="Y5" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="Z5" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="AA5" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="AB5" s="3" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -1293,6 +1372,18 @@
           <t>Habilita MAN_A</t>
         </is>
       </c>
+      <c r="Y6" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="Z6" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="AA6" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="AB6" s="3" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -1367,6 +1458,18 @@
       <c r="V7" s="2" t="n"/>
       <c r="W7" s="2" t="n"/>
       <c r="X7" s="2" t="inlineStr"/>
+      <c r="Y7" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="Z7" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="AA7" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="AB7" s="3" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -1441,6 +1544,18 @@
       <c r="V8" s="2" t="n"/>
       <c r="W8" s="2" t="n"/>
       <c r="X8" s="2" t="inlineStr"/>
+      <c r="Y8" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="Z8" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="AA8" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="AB8" s="3" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -1515,6 +1630,18 @@
       <c r="V9" s="2" t="n"/>
       <c r="W9" s="2" t="n"/>
       <c r="X9" s="2" t="inlineStr"/>
+      <c r="Y9" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="Z9" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="AA9" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="AB9" s="3" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -1589,6 +1716,18 @@
       <c r="V10" s="2" t="n"/>
       <c r="W10" s="2" t="n"/>
       <c r="X10" s="2" t="inlineStr"/>
+      <c r="Y10" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="Z10" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="AA10" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="AB10" s="3" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -1671,6 +1810,18 @@
           <t>Condición O</t>
         </is>
       </c>
+      <c r="Y11" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="Z11" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="AA11" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="AB11" s="3" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -1737,6 +1888,18 @@
       <c r="V12" s="2" t="n"/>
       <c r="W12" s="2" t="n"/>
       <c r="X12" s="2" t="inlineStr"/>
+      <c r="Y12" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="Z12" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="AA12" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="AB12" s="3" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -1815,6 +1978,18 @@
           <t>Si MAN_A ya se usó, el texto queda raro: revisar en el paso 9</t>
         </is>
       </c>
+      <c r="Y13" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="Z13" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="AA13" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="AB13" s="3" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -1889,6 +2064,18 @@
       <c r="V14" s="2" t="n"/>
       <c r="W14" s="2" t="n"/>
       <c r="X14" s="2" t="inlineStr"/>
+      <c r="Y14" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="Z14" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="AA14" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="AB14" s="3" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -1955,6 +2142,18 @@
       <c r="V15" s="2" t="n"/>
       <c r="W15" s="2" t="n"/>
       <c r="X15" s="2" t="inlineStr"/>
+      <c r="Y15" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="Z15" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="AA15" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="AB15" s="3" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -2027,6 +2226,18 @@
       <c r="V16" s="2" t="n"/>
       <c r="W16" s="2" t="n"/>
       <c r="X16" s="2" t="inlineStr"/>
+      <c r="Y16" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="Z16" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="AA16" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="AB16" s="3" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -2099,6 +2310,18 @@
       <c r="V17" s="2" t="n"/>
       <c r="W17" s="2" t="n"/>
       <c r="X17" s="2" t="inlineStr"/>
+      <c r="Y17" s="3" t="n">
+        <v>13</v>
+      </c>
+      <c r="Z17" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="AA17" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="AB17" s="3" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -2171,6 +2394,18 @@
       <c r="V18" s="2" t="n"/>
       <c r="W18" s="2" t="n"/>
       <c r="X18" s="2" t="inlineStr"/>
+      <c r="Y18" s="3" t="n">
+        <v>16</v>
+      </c>
+      <c r="Z18" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="AA18" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="AB18" s="3" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -2249,6 +2484,18 @@
       <c r="V19" s="2" t="n"/>
       <c r="W19" s="2" t="n"/>
       <c r="X19" s="2" t="inlineStr"/>
+      <c r="Y19" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="Z19" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="AA19" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="AB19" s="3" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -2321,6 +2568,18 @@
       <c r="V20" s="2" t="n"/>
       <c r="W20" s="2" t="n"/>
       <c r="X20" s="2" t="inlineStr"/>
+      <c r="Y20" s="3" t="n">
+        <v>16</v>
+      </c>
+      <c r="Z20" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="AA20" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="AB20" s="3" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -2387,6 +2646,18 @@
       <c r="V21" s="2" t="n"/>
       <c r="W21" s="2" t="n"/>
       <c r="X21" s="2" t="inlineStr"/>
+      <c r="Y21" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="Z21" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="AA21" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="AB21" s="3" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -2459,6 +2730,18 @@
       <c r="V22" s="2" t="n"/>
       <c r="W22" s="2" t="n"/>
       <c r="X22" s="2" t="inlineStr"/>
+      <c r="Y22" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="Z22" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="AA22" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="AB22" s="3" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -2531,6 +2814,18 @@
       <c r="V23" s="2" t="n"/>
       <c r="W23" s="2" t="n"/>
       <c r="X23" s="2" t="inlineStr"/>
+      <c r="Y23" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="Z23" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="AA23" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="AB23" s="3" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -2601,6 +2896,18 @@
           <t>Activa COM_M (tijera del pasado)</t>
         </is>
       </c>
+      <c r="Y24" s="3" t="n">
+        <v>13</v>
+      </c>
+      <c r="Z24" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="AA24" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="AB24" s="3" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -2667,6 +2974,18 @@
       <c r="V25" s="2" t="n"/>
       <c r="W25" s="2" t="n"/>
       <c r="X25" s="2" t="inlineStr"/>
+      <c r="Y25" s="3" t="n">
+        <v>16</v>
+      </c>
+      <c r="Z25" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="AA25" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="AB25" s="3" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -2751,6 +3070,18 @@
       <c r="V26" s="2" t="n"/>
       <c r="W26" s="2" t="n"/>
       <c r="X26" s="2" t="inlineStr"/>
+      <c r="Y26" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="Z26" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="AA26" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="AB26" s="3" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -2828,6 +3159,18 @@
         <is>
           <t>Forzada al entrar (antes Costo 4 + diálogo al entrar). Su Usado activa la tijera del presente y del futuro</t>
         </is>
+      </c>
+      <c r="Y27" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="Z27" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="AA27" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="AB27" s="3" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="28">
@@ -2901,6 +3244,18 @@
           <t>Solo visual</t>
         </is>
       </c>
+      <c r="Y28" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="Z28" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="AA28" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="AB28" s="3" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -2996,6 +3351,18 @@
         <is>
           <t>Usa 4 disparadores (el modelo de 02 tenía 3)</t>
         </is>
+      </c>
+      <c r="Y29" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="Z29" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="AA29" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="AB29" s="3" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="30">
@@ -3069,6 +3436,18 @@
           <t>Solo visual</t>
         </is>
       </c>
+      <c r="Y30" s="3" t="n">
+        <v>9</v>
+      </c>
+      <c r="Z30" s="3" t="n">
+        <v>9</v>
+      </c>
+      <c r="AA30" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="AB30" s="3" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -3145,6 +3524,18 @@
           <t>Va en COM porque se interactúa desde ahí (el 06 la ponía en SCO)</t>
         </is>
       </c>
+      <c r="Y31" s="3" t="n">
+        <v>17</v>
+      </c>
+      <c r="Z31" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="AA31" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="AB31" s="3" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -3217,6 +3608,18 @@
       <c r="V32" s="2" t="n"/>
       <c r="W32" s="2" t="n"/>
       <c r="X32" s="2" t="inlineStr"/>
+      <c r="Y32" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="Z32" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="AA32" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="AB32" s="3" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -3283,6 +3686,18 @@
       <c r="V33" s="2" t="n"/>
       <c r="W33" s="2" t="n"/>
       <c r="X33" s="2" t="inlineStr"/>
+      <c r="Y33" s="3" t="n">
+        <v>19</v>
+      </c>
+      <c r="Z33" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="AA33" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="AB33" s="3" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -3355,6 +3770,18 @@
       <c r="V34" s="2" t="n"/>
       <c r="W34" s="2" t="n"/>
       <c r="X34" s="2" t="inlineStr"/>
+      <c r="Y34" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="Z34" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="AA34" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="AB34" s="3" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
@@ -3431,6 +3858,18 @@
           <t>Activa SCO_J y SCO_O; desdibuja SCO_I</t>
         </is>
       </c>
+      <c r="Y35" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="Z35" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="AA35" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="AB35" s="3" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -3506,6 +3945,18 @@
         <is>
           <t>Beta</t>
         </is>
+      </c>
+      <c r="Y36" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="Z36" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="AA36" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="AB36" s="3" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="37">
@@ -3577,6 +4028,18 @@
           <t>Beta</t>
         </is>
       </c>
+      <c r="Y37" s="3" t="n">
+        <v>15</v>
+      </c>
+      <c r="Z37" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="AA37" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="AB37" s="3" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -3649,6 +4112,18 @@
       <c r="V38" s="2" t="n"/>
       <c r="W38" s="2" t="n"/>
       <c r="X38" s="2" t="inlineStr"/>
+      <c r="Y38" s="3" t="n">
+        <v>12</v>
+      </c>
+      <c r="Z38" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="AA38" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="AB38" s="3" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
@@ -3721,6 +4196,18 @@
       <c r="V39" s="2" t="n"/>
       <c r="W39" s="2" t="n"/>
       <c r="X39" s="2" t="inlineStr"/>
+      <c r="Y39" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="Z39" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="AA39" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="AB39" s="3" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -3787,6 +4274,18 @@
       <c r="V40" s="2" t="n"/>
       <c r="W40" s="2" t="n"/>
       <c r="X40" s="2" t="inlineStr"/>
+      <c r="Y40" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="Z40" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="AA40" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="AB40" s="3" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
@@ -3867,6 +4366,18 @@
       <c r="V41" s="2" t="n"/>
       <c r="W41" s="2" t="n"/>
       <c r="X41" s="2" t="inlineStr"/>
+      <c r="Y41" s="3" t="n">
+        <v>9</v>
+      </c>
+      <c r="Z41" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="AA41" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="AB41" s="3" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
@@ -3939,6 +4450,18 @@
       <c r="V42" s="2" t="n"/>
       <c r="W42" s="2" t="n"/>
       <c r="X42" s="2" t="inlineStr"/>
+      <c r="Y42" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="Z42" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="AA42" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="AB42" s="3" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
@@ -4014,6 +4537,18 @@
         <is>
           <t>Beta</t>
         </is>
+      </c>
+      <c r="Y43" s="3" t="n">
+        <v>18</v>
+      </c>
+      <c r="Z43" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="AA43" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="AB43" s="3" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="44">
@@ -4085,6 +4620,18 @@
           <t>Beta</t>
         </is>
       </c>
+      <c r="Y44" s="3" t="n">
+        <v>16</v>
+      </c>
+      <c r="Z44" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="AA44" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="AB44" s="3" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
@@ -4151,6 +4698,18 @@
       <c r="V45" s="2" t="n"/>
       <c r="W45" s="2" t="n"/>
       <c r="X45" s="2" t="inlineStr"/>
+      <c r="Y45" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="Z45" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="AA45" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="AB45" s="3" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
@@ -4231,6 +4790,18 @@
       <c r="V46" s="2" t="n"/>
       <c r="W46" s="2" t="n"/>
       <c r="X46" s="2" t="inlineStr"/>
+      <c r="Y46" s="3" t="n">
+        <v>9</v>
+      </c>
+      <c r="Z46" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="AA46" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="AB46" s="3" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
@@ -4301,6 +4872,18 @@
           <t>Beta</t>
         </is>
       </c>
+      <c r="Y47" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="Z47" s="3" t="n">
+        <v>9</v>
+      </c>
+      <c r="AA47" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="AB47" s="3" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
@@ -4370,6 +4953,18 @@
         <is>
           <t>Beta</t>
         </is>
+      </c>
+      <c r="Y48" s="3" t="n">
+        <v>19</v>
+      </c>
+      <c r="Z48" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="AA48" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="AB48" s="3" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="49">
@@ -4443,6 +5038,18 @@
           <t>Solo visual</t>
         </is>
       </c>
+      <c r="Y49" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="Z49" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="AA49" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="AB49" s="3" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
@@ -4513,6 +5120,18 @@
           <t>[Propuesta] pendiente de confirmar</t>
         </is>
       </c>
+      <c r="Y50" s="3" t="n">
+        <v>21</v>
+      </c>
+      <c r="Z50" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="AA50" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="AB50" s="3" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
@@ -4585,6 +5204,18 @@
       <c r="V51" s="2" t="n"/>
       <c r="W51" s="2" t="n"/>
       <c r="X51" s="2" t="inlineStr"/>
+      <c r="Y51" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="Z51" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA51" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="AB51" s="3" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
@@ -4651,6 +5282,18 @@
       <c r="V52" s="2" t="n"/>
       <c r="W52" s="2" t="n"/>
       <c r="X52" s="2" t="inlineStr"/>
+      <c r="Y52" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="Z52" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="AA52" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="AB52" s="3" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
@@ -4723,6 +5366,18 @@
       <c r="V53" s="2" t="n"/>
       <c r="W53" s="2" t="n"/>
       <c r="X53" s="2" t="inlineStr"/>
+      <c r="Y53" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="Z53" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA53" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="AB53" s="3" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
@@ -4789,6 +5444,18 @@
       <c r="V54" s="2" t="n"/>
       <c r="W54" s="2" t="n"/>
       <c r="X54" s="2" t="inlineStr"/>
+      <c r="Y54" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="Z54" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA54" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="AB54" s="3" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
@@ -4855,9 +5522,21 @@
       <c r="V55" s="2" t="n"/>
       <c r="W55" s="2" t="n"/>
       <c r="X55" s="2" t="inlineStr"/>
+      <c r="Y55" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="Z55" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="AA55" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="AB55" s="3" t="n">
+        <v>1</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:X55"/>
+  <autoFilter ref="A1:AB55"/>
   <dataValidations count="8">
     <dataValidation sqref="F2:F300" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"pasado,presente,futuro"</formula1>

</xml_diff>

<commit_message>
Paso 4: objetos con nombre, interacción, diálogos, zoom y menú de pausa
</commit_message>
<xml_diff>
--- a/planilla/contenido_alfa.xlsx
+++ b/planilla/contenido_alfa.xlsx
@@ -21,7 +21,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'LEEME'!$A$1:$A$17</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'objetos'!$A$1:$AB$55</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'objetos'!$A$1:$AC$55</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'salas'!$A$1:$I$5</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'guion'!$A$1:$E$13</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'textos'!$A$1:$D$68</definedName>
@@ -456,7 +456,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A19"/>
+  <dimension ref="A1:A20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="140" customWidth="1" min="1" max="1"/>
@@ -584,6 +584,13 @@
       <c r="A19" s="3" t="inlineStr">
         <is>
           <t>Posición de cada objeto: x, y, ancho, alto en tiles de 16 px, desde la esquina de arriba a la izquierda de la sala (la pared ocupa medio tile). Las conversaciones de NORA comparten el lugar de la consola.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="3" t="inlineStr">
+        <is>
+          <t>Nombre: lo que ve el jugador al acercarse ("E: investigar Radio"). Sin spoilers: describe lo que se ve, nunca el tiempo ni la causa.</t>
         </is>
       </c>
     </row>
@@ -796,7 +803,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AB55"/>
+  <dimension ref="A1:AC55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -827,6 +834,7 @@
     <col width="6" customWidth="1" min="26" max="26"/>
     <col width="6" customWidth="1" min="27" max="27"/>
     <col width="6" customWidth="1" min="28" max="28"/>
+    <col width="24" customWidth="1" min="29" max="29"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -968,6 +976,11 @@
       <c r="AB1" s="4" t="inlineStr">
         <is>
           <t>alto</t>
+        </is>
+      </c>
+      <c r="AC1" s="4" t="inlineStr">
+        <is>
+          <t>nombre</t>
         </is>
       </c>
     </row>
@@ -1067,6 +1080,11 @@
       </c>
       <c r="AB2" s="3" t="n">
         <v>1</v>
+      </c>
+      <c r="AC2" s="3" t="inlineStr">
+        <is>
+          <t>Panel eléctrico</t>
+        </is>
       </c>
     </row>
     <row r="3">
@@ -1146,6 +1164,11 @@
       <c r="AB3" s="3" t="n">
         <v>1</v>
       </c>
+      <c r="AC3" s="3" t="inlineStr">
+        <is>
+          <t>Consola de NORA</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -1224,6 +1247,11 @@
       <c r="AB4" s="3" t="n">
         <v>1</v>
       </c>
+      <c r="AC4" s="3" t="inlineStr">
+        <is>
+          <t>Consola de NORA</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -1302,6 +1330,11 @@
       <c r="AB5" s="3" t="n">
         <v>1</v>
       </c>
+      <c r="AC5" s="3" t="inlineStr">
+        <is>
+          <t>Consola de NORA</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -1383,6 +1416,11 @@
       </c>
       <c r="AB6" s="3" t="n">
         <v>1</v>
+      </c>
+      <c r="AC6" s="3" t="inlineStr">
+        <is>
+          <t>Consola de NORA</t>
+        </is>
       </c>
     </row>
     <row r="7">
@@ -1470,6 +1508,11 @@
       <c r="AB7" s="3" t="n">
         <v>1</v>
       </c>
+      <c r="AC7" s="3" t="inlineStr">
+        <is>
+          <t>Consola de NORA</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -1556,6 +1599,11 @@
       <c r="AB8" s="3" t="n">
         <v>1</v>
       </c>
+      <c r="AC8" s="3" t="inlineStr">
+        <is>
+          <t>Consola de NORA</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -1642,6 +1690,11 @@
       <c r="AB9" s="3" t="n">
         <v>1</v>
       </c>
+      <c r="AC9" s="3" t="inlineStr">
+        <is>
+          <t>Consola de NORA</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -1728,6 +1781,11 @@
       <c r="AB10" s="3" t="n">
         <v>1</v>
       </c>
+      <c r="AC10" s="3" t="inlineStr">
+        <is>
+          <t>Consola de NORA</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -1821,6 +1879,11 @@
       </c>
       <c r="AB11" s="3" t="n">
         <v>1</v>
+      </c>
+      <c r="AC11" s="3" t="inlineStr">
+        <is>
+          <t>Consola de NORA</t>
+        </is>
       </c>
     </row>
     <row r="12">
@@ -1900,6 +1963,11 @@
       <c r="AB12" s="3" t="n">
         <v>1</v>
       </c>
+      <c r="AC12" s="3" t="inlineStr">
+        <is>
+          <t>Consola de NORA</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -1989,6 +2057,11 @@
       </c>
       <c r="AB13" s="3" t="n">
         <v>1</v>
+      </c>
+      <c r="AC13" s="3" t="inlineStr">
+        <is>
+          <t>Consola de NORA</t>
+        </is>
       </c>
     </row>
     <row r="14">
@@ -2076,6 +2149,11 @@
       <c r="AB14" s="3" t="n">
         <v>1</v>
       </c>
+      <c r="AC14" s="3" t="inlineStr">
+        <is>
+          <t>Consola de NORA</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -2154,6 +2232,11 @@
       <c r="AB15" s="3" t="n">
         <v>1</v>
       </c>
+      <c r="AC15" s="3" t="inlineStr">
+        <is>
+          <t>Taza de café</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -2238,6 +2321,11 @@
       <c r="AB16" s="3" t="n">
         <v>1</v>
       </c>
+      <c r="AC16" s="3" t="inlineStr">
+        <is>
+          <t>Consola de radio</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -2322,6 +2410,11 @@
       <c r="AB17" s="3" t="n">
         <v>1</v>
       </c>
+      <c r="AC17" s="3" t="inlineStr">
+        <is>
+          <t>Panel de herramientas</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -2406,6 +2499,11 @@
       <c r="AB18" s="3" t="n">
         <v>2</v>
       </c>
+      <c r="AC18" s="3" t="inlineStr">
+        <is>
+          <t>Lista de turnos</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -2495,6 +2593,11 @@
       </c>
       <c r="AB19" s="3" t="n">
         <v>1</v>
+      </c>
+      <c r="AC19" s="3" t="inlineStr">
+        <is>
+          <t>Radio</t>
+        </is>
       </c>
     </row>
     <row r="20">
@@ -2579,6 +2682,11 @@
       </c>
       <c r="AB20" s="3" t="n">
         <v>2</v>
+      </c>
+      <c r="AC20" s="3" t="inlineStr">
+        <is>
+          <t>Plano de evacuación</t>
+        </is>
       </c>
     </row>
     <row r="21">
@@ -2658,6 +2766,11 @@
       <c r="AB21" s="3" t="n">
         <v>1</v>
       </c>
+      <c r="AC21" s="3" t="inlineStr">
+        <is>
+          <t>Hojas de protocolo</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -2742,6 +2855,11 @@
       <c r="AB22" s="3" t="n">
         <v>1</v>
       </c>
+      <c r="AC22" s="3" t="inlineStr">
+        <is>
+          <t>Registro de transmisiones</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -2826,6 +2944,11 @@
       <c r="AB23" s="3" t="n">
         <v>1</v>
       </c>
+      <c r="AC23" s="3" t="inlineStr">
+        <is>
+          <t>Consola de radio</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -2907,6 +3030,11 @@
       </c>
       <c r="AB24" s="3" t="n">
         <v>1</v>
+      </c>
+      <c r="AC24" s="3" t="inlineStr">
+        <is>
+          <t>Panel de herramientas</t>
+        </is>
       </c>
     </row>
     <row r="25">
@@ -2986,6 +3114,11 @@
       <c r="AB25" s="3" t="n">
         <v>2</v>
       </c>
+      <c r="AC25" s="3" t="inlineStr">
+        <is>
+          <t>Plano de evacuación</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -3082,6 +3215,11 @@
       <c r="AB26" s="3" t="n">
         <v>1</v>
       </c>
+      <c r="AC26" s="3" t="inlineStr">
+        <is>
+          <t>Nota en la radio</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -3171,6 +3309,11 @@
       </c>
       <c r="AB27" s="3" t="n">
         <v>1</v>
+      </c>
+      <c r="AC27" s="3" t="inlineStr">
+        <is>
+          <t>Tijera</t>
+        </is>
       </c>
     </row>
     <row r="28">
@@ -3256,6 +3399,11 @@
       <c r="AB28" s="3" t="n">
         <v>1</v>
       </c>
+      <c r="AC28" s="3" t="inlineStr">
+        <is>
+          <t>Tijera</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -3363,6 +3511,11 @@
       </c>
       <c r="AB29" s="3" t="n">
         <v>1</v>
+      </c>
+      <c r="AC29" s="3" t="inlineStr">
+        <is>
+          <t>Tijera</t>
+        </is>
       </c>
     </row>
     <row r="30">
@@ -3448,6 +3601,11 @@
       <c r="AB30" s="3" t="n">
         <v>1</v>
       </c>
+      <c r="AC30" s="3" t="inlineStr">
+        <is>
+          <t>Hoja rota</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -3535,6 +3693,11 @@
       </c>
       <c r="AB31" s="3" t="n">
         <v>2</v>
+      </c>
+      <c r="AC31" s="3" t="inlineStr">
+        <is>
+          <t>Puerta de la sala común</t>
+        </is>
       </c>
     </row>
     <row r="32">
@@ -3619,6 +3782,11 @@
       </c>
       <c r="AB32" s="3" t="n">
         <v>2</v>
+      </c>
+      <c r="AC32" s="3" t="inlineStr">
+        <is>
+          <t>Mesa larga</t>
+        </is>
       </c>
     </row>
     <row r="33">
@@ -3698,6 +3866,11 @@
       <c r="AB33" s="3" t="n">
         <v>2</v>
       </c>
+      <c r="AC33" s="3" t="inlineStr">
+        <is>
+          <t>Dispensador de agua</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -3782,6 +3955,11 @@
       <c r="AB34" s="3" t="n">
         <v>1</v>
       </c>
+      <c r="AC34" s="3" t="inlineStr">
+        <is>
+          <t>Pizarra de turnos</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
@@ -3870,6 +4048,11 @@
       <c r="AB35" s="3" t="n">
         <v>1</v>
       </c>
+      <c r="AC35" s="3" t="inlineStr">
+        <is>
+          <t>Taza con mi nombre</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -3957,6 +4140,11 @@
       </c>
       <c r="AB36" s="3" t="n">
         <v>1</v>
+      </c>
+      <c r="AC36" s="3" t="inlineStr">
+        <is>
+          <t>Calendario</t>
+        </is>
       </c>
     </row>
     <row r="37">
@@ -4040,6 +4228,11 @@
       <c r="AB37" s="3" t="n">
         <v>1</v>
       </c>
+      <c r="AC37" s="3" t="inlineStr">
+        <is>
+          <t>Foto de la tripulación</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -4124,6 +4317,11 @@
       <c r="AB38" s="3" t="n">
         <v>1</v>
       </c>
+      <c r="AC38" s="3" t="inlineStr">
+        <is>
+          <t>Partida de cartas</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
@@ -4207,6 +4405,11 @@
       </c>
       <c r="AB39" s="3" t="n">
         <v>1</v>
+      </c>
+      <c r="AC39" s="3" t="inlineStr">
+        <is>
+          <t>Silla volcada</t>
+        </is>
       </c>
     </row>
     <row r="40">
@@ -4286,6 +4489,11 @@
       <c r="AB40" s="3" t="n">
         <v>1</v>
       </c>
+      <c r="AC40" s="3" t="inlineStr">
+        <is>
+          <t>Taza con mi nombre</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
@@ -4378,6 +4586,11 @@
       <c r="AB41" s="3" t="n">
         <v>1</v>
       </c>
+      <c r="AC41" s="3" t="inlineStr">
+        <is>
+          <t>Taza sobre la mesa</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
@@ -4462,6 +4675,11 @@
       <c r="AB42" s="3" t="n">
         <v>1</v>
       </c>
+      <c r="AC42" s="3" t="inlineStr">
+        <is>
+          <t>Pizarra de turnos</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
@@ -4549,6 +4767,11 @@
       </c>
       <c r="AB43" s="3" t="n">
         <v>1</v>
+      </c>
+      <c r="AC43" s="3" t="inlineStr">
+        <is>
+          <t>Reloj de pared</t>
+        </is>
       </c>
     </row>
     <row r="44">
@@ -4631,6 +4854,11 @@
       </c>
       <c r="AB44" s="3" t="n">
         <v>1</v>
+      </c>
+      <c r="AC44" s="3" t="inlineStr">
+        <is>
+          <t>Chaqueta</t>
+        </is>
       </c>
     </row>
     <row r="45">
@@ -4710,6 +4938,11 @@
       <c r="AB45" s="3" t="n">
         <v>2</v>
       </c>
+      <c r="AC45" s="3" t="inlineStr">
+        <is>
+          <t>Mesa partida</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
@@ -4802,6 +5035,11 @@
       <c r="AB46" s="3" t="n">
         <v>1</v>
       </c>
+      <c r="AC46" s="3" t="inlineStr">
+        <is>
+          <t>Taza rota</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
@@ -4884,6 +5122,11 @@
       <c r="AB47" s="3" t="n">
         <v>1</v>
       </c>
+      <c r="AC47" s="3" t="inlineStr">
+        <is>
+          <t>Calendario caído</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
@@ -4965,6 +5208,11 @@
       </c>
       <c r="AB48" s="3" t="n">
         <v>2</v>
+      </c>
+      <c r="AC48" s="3" t="inlineStr">
+        <is>
+          <t>Dispensador de agua</t>
+        </is>
       </c>
     </row>
     <row r="49">
@@ -5050,6 +5298,11 @@
       <c r="AB49" s="3" t="n">
         <v>1</v>
       </c>
+      <c r="AC49" s="3" t="inlineStr">
+        <is>
+          <t>Silla</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
@@ -5132,6 +5385,11 @@
       <c r="AB50" s="3" t="n">
         <v>2</v>
       </c>
+      <c r="AC50" s="3" t="inlineStr">
+        <is>
+          <t>Puertas hacia el resto de la nave</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
@@ -5215,6 +5473,11 @@
       </c>
       <c r="AB51" s="3" t="n">
         <v>1</v>
+      </c>
+      <c r="AC51" s="3" t="inlineStr">
+        <is>
+          <t>Puerta</t>
+        </is>
       </c>
     </row>
     <row r="52">
@@ -5294,6 +5557,11 @@
       <c r="AB52" s="3" t="n">
         <v>1</v>
       </c>
+      <c r="AC52" s="3" t="inlineStr">
+        <is>
+          <t>Soporte de placa</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
@@ -5377,6 +5645,11 @@
       </c>
       <c r="AB53" s="3" t="n">
         <v>1</v>
+      </c>
+      <c r="AC53" s="3" t="inlineStr">
+        <is>
+          <t>Puerta</t>
+        </is>
       </c>
     </row>
     <row r="54">
@@ -5456,6 +5729,11 @@
       <c r="AB54" s="3" t="n">
         <v>1</v>
       </c>
+      <c r="AC54" s="3" t="inlineStr">
+        <is>
+          <t>Puerta</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
@@ -5534,9 +5812,14 @@
       <c r="AB55" s="3" t="n">
         <v>1</v>
       </c>
+      <c r="AC55" s="3" t="inlineStr">
+        <is>
+          <t>Polvo junto a la puerta</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AB55"/>
+  <autoFilter ref="A1:AC55"/>
   <dataValidations count="8">
     <dataValidation sqref="F2:F300" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"pasado,presente,futuro"</formula1>

</xml_diff>

<commit_message>
Paso 5 y correciones varias
</commit_message>
<xml_diff>
--- a/planilla/contenido_alfa.xlsx
+++ b/planilla/contenido_alfa.xlsx
@@ -12,24 +12,25 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="salas" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="guion" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="conexiones" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="textos" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="anotaciones" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="items" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="audios" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="eventos" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="config" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="muebles" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="textos" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="anotaciones" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="items" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="audios" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="eventos" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="config" sheetId="12" state="visible" r:id="rId12"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'LEEME'!$A$1:$A$17</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'objetos'!$A$1:$AC$55</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'salas'!$A$1:$I$5</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'guion'!$A$1:$E$13</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'textos'!$A$1:$D$68</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'anotaciones'!$A$1:$B$21</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'items'!$A$1:$C$2</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'audios'!$A$1:$B$3</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'eventos'!$A$1:$B$3</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'config'!$A$1:$C$7</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'textos'!$A$1:$D$68</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'anotaciones'!$A$1:$B$21</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'items'!$A$1:$C$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'audios'!$A$1:$B$3</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'eventos'!$A$1:$B$3</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'config'!$A$1:$C$7</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -456,7 +457,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A20"/>
+  <dimension ref="A1:A28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="140" customWidth="1" min="1" max="1"/>
@@ -591,6 +592,55 @@
       <c r="A20" s="3" t="inlineStr">
         <is>
           <t>Nombre: lo que ve el jugador al acercarse ("E: investigar Radio"). Sin spoilers: describe lo que se ve, nunca el tiempo ni la causa.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Agregado el 21/10/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>turnoMax (objetos): último turno en que el objeto existe (vacío = sin límite). oculto = sí: no se dibuja; sirve como punto al que camina una cinemática.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Forzada: el personaje camina solo hasta el objeto (cinemática) y recién ahí sale el diálogo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Conexiones: vuelta_gratis = sí → ir de 'hasta' a 'desde' no cuesta energía.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Muebles: hoja propia. Son fijos: se dibujan igual en todos los tiempos (mesas, sillas, paneles). Solo cambian los objetos que están encima.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Textos SIS_…: los usa el código (descansar con NORA, quedarse sin energía), no un objeto.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Muebles: solido = sí → tiene colisión (se rodea; nunca tapar el camino entre puertas). en_futuro: caído / roto → en el futuro se dibuja así. Un mueble nunca desaparece.</t>
         </is>
       </c>
     </row>
@@ -609,8 +659,8 @@
   <dimension ref="A1:B3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="18" customWidth="1" min="1" max="1"/>
-    <col width="80" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="60" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -628,24 +678,24 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>arreglo_com</t>
+          <t>estatica</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Comunicaciones pasa a poder tener luz máxima (3).</t>
+          <t>Estática de radio (placeholder)</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>desbloquear_SCO</t>
+          <t>chisporroteo</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Desbloquea la sala común. Queda con luz 0.</t>
+          <t>Chisporroteo eléctrico (placeholder)</t>
         </is>
       </c>
     </row>
@@ -656,6 +706,61 @@
 </file>
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="80" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>descripcion</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>arreglo_com</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Comunicaciones pasa a poder tener luz máxima (3).</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>desbloquear_SCO</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Desbloquea la sala común. Queda con luz 0.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:B3"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -803,7 +908,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AC55"/>
+  <dimension ref="A1:AE57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -835,6 +940,8 @@
     <col width="6" customWidth="1" min="27" max="27"/>
     <col width="6" customWidth="1" min="28" max="28"/>
     <col width="24" customWidth="1" min="29" max="29"/>
+    <col width="10" customWidth="1" min="30" max="30"/>
+    <col width="10" customWidth="1" min="31" max="31"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -981,6 +1088,16 @@
       <c r="AC1" s="4" t="inlineStr">
         <is>
           <t>nombre</t>
+        </is>
+      </c>
+      <c r="AD1" s="1" t="inlineStr">
+        <is>
+          <t>turnoMax</t>
+        </is>
+      </c>
+      <c r="AE1" s="1" t="inlineStr">
+        <is>
+          <t>oculto</t>
         </is>
       </c>
     </row>
@@ -1212,12 +1329,20 @@
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>sí</t>
         </is>
       </c>
       <c r="K4" s="2" t="n"/>
-      <c r="L4" s="2" t="n"/>
-      <c r="M4" s="2" t="n"/>
+      <c r="L4" s="2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="M4" s="2" t="inlineStr">
+        <is>
+          <t>MAN_N1.Usado</t>
+        </is>
+      </c>
       <c r="N4" s="2" t="n"/>
       <c r="O4" s="2" t="n"/>
       <c r="P4" s="2" t="n">
@@ -1234,7 +1359,11 @@
       <c r="U4" s="2" t="n"/>
       <c r="V4" s="2" t="n"/>
       <c r="W4" s="2" t="n"/>
-      <c r="X4" s="2" t="inlineStr"/>
+      <c r="X4" s="2" t="inlineStr">
+        <is>
+          <t>T1 obligatoria, en cadena después de N1</t>
+        </is>
+      </c>
       <c r="Y4" s="3" t="n">
         <v>8</v>
       </c>
@@ -1295,12 +1424,20 @@
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>sí</t>
         </is>
       </c>
       <c r="K5" s="2" t="n"/>
-      <c r="L5" s="2" t="n"/>
-      <c r="M5" s="2" t="n"/>
+      <c r="L5" s="2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="M5" s="2" t="inlineStr">
+        <is>
+          <t>MAN_N2.Usado</t>
+        </is>
+      </c>
       <c r="N5" s="2" t="n"/>
       <c r="O5" s="2" t="n"/>
       <c r="P5" s="2" t="n">
@@ -1317,7 +1454,11 @@
       <c r="U5" s="2" t="n"/>
       <c r="V5" s="2" t="n"/>
       <c r="W5" s="2" t="n"/>
-      <c r="X5" s="2" t="inlineStr"/>
+      <c r="X5" s="2" t="inlineStr">
+        <is>
+          <t>T1 obligatoria, en cadena después de N2</t>
+        </is>
+      </c>
       <c r="Y5" s="3" t="n">
         <v>8</v>
       </c>
@@ -1378,12 +1519,20 @@
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>sí</t>
         </is>
       </c>
       <c r="K6" s="2" t="n"/>
-      <c r="L6" s="2" t="n"/>
-      <c r="M6" s="2" t="n"/>
+      <c r="L6" s="2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="M6" s="2" t="inlineStr">
+        <is>
+          <t>MAN_N3.Usado</t>
+        </is>
+      </c>
       <c r="N6" s="2" t="n"/>
       <c r="O6" s="2" t="n"/>
       <c r="P6" s="2" t="n">
@@ -1402,7 +1551,7 @@
       <c r="W6" s="2" t="n"/>
       <c r="X6" s="2" t="inlineStr">
         <is>
-          <t>Habilita MAN_A</t>
+          <t>T1 obligatoria, en cadena después de N3</t>
         </is>
       </c>
       <c r="Y6" s="3" t="n">
@@ -3244,7 +3393,7 @@
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>Tijera sobre la mesa (se observa, nunca se agarra)</t>
+          <t>Tijera sobre la mesa (el personaje ya tiene la del futuro en el bolsillo)</t>
         </is>
       </c>
       <c r="F27" s="2" t="inlineStr">
@@ -3263,7 +3412,7 @@
       </c>
       <c r="J27" s="2" t="inlineStr">
         <is>
-          <t>sí</t>
+          <t>no</t>
         </is>
       </c>
       <c r="K27" s="2" t="n"/>
@@ -3274,7 +3423,7 @@
       </c>
       <c r="M27" s="2" t="inlineStr">
         <is>
-          <t>COM_J.Usado</t>
+          <t>COM_O.Usado</t>
         </is>
       </c>
       <c r="N27" s="2" t="n"/>
@@ -3287,15 +3436,27 @@
           <t>T_COM_M</t>
         </is>
       </c>
-      <c r="R27" s="2" t="n"/>
-      <c r="S27" s="2" t="n"/>
-      <c r="T27" s="2" t="n"/>
-      <c r="U27" s="2" t="n"/>
+      <c r="R27" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="S27" s="2" t="inlineStr">
+        <is>
+          <t>A_COM_M</t>
+        </is>
+      </c>
+      <c r="T27" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="U27" s="2" t="inlineStr">
+        <is>
+          <t>COM_S</t>
+        </is>
+      </c>
       <c r="V27" s="2" t="n"/>
       <c r="W27" s="2" t="n"/>
       <c r="X27" s="2" t="inlineStr">
         <is>
-          <t>Forzada al entrar (antes Costo 4 + diálogo al entrar). Su Usado activa la tijera del presente y del futuro</t>
+          <t>Opcional (T9). Investigarla da la confusión; no se la lleva y queda a la vista. Cancela el diálogo obligatorio del presente (COM_S)</t>
         </is>
       </c>
       <c r="Y27" s="3" t="n">
@@ -3339,7 +3500,7 @@
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>Tijera sobre la mesa</t>
+          <t>Tijera sobre la mesa (la otra está en el bolsillo)</t>
         </is>
       </c>
       <c r="F28" s="2" t="inlineStr">
@@ -3348,7 +3509,7 @@
         </is>
       </c>
       <c r="G28" s="2" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="H28" s="2" t="n">
         <v>1</v>
@@ -3369,7 +3530,7 @@
       </c>
       <c r="M28" s="2" t="inlineStr">
         <is>
-          <t>COM_M.Usado</t>
+          <t>COM_O.Usado</t>
         </is>
       </c>
       <c r="N28" s="2" t="n"/>
@@ -3384,7 +3545,7 @@
       <c r="W28" s="2" t="n"/>
       <c r="X28" s="2" t="inlineStr">
         <is>
-          <t>Solo visual</t>
+          <t>Solo visual: siempre a la vista en el presente después de agarrar la del futuro</t>
         </is>
       </c>
       <c r="Y28" s="3" t="n">
@@ -3437,7 +3598,7 @@
         </is>
       </c>
       <c r="G29" s="2" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="H29" s="2" t="n">
         <v>1</v>
@@ -3451,16 +3612,8 @@
         </is>
       </c>
       <c r="K29" s="2" t="n"/>
-      <c r="L29" s="2" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="M29" s="2" t="inlineStr">
-        <is>
-          <t>COM_M.Usado</t>
-        </is>
-      </c>
+      <c r="L29" s="2" t="n"/>
+      <c r="M29" s="2" t="n"/>
       <c r="N29" s="2" t="n"/>
       <c r="O29" s="2" t="n"/>
       <c r="P29" s="2" t="n">
@@ -3497,7 +3650,7 @@
       </c>
       <c r="X29" s="2" t="inlineStr">
         <is>
-          <t>Usa 4 disparadores (el modelo de 02 tenía 3)</t>
+          <t>Primer futuro (T7): se agarra sola (cinemática). Se desdibuja: en el futuro ya no vuelve a estar</t>
         </is>
       </c>
       <c r="Y29" s="3" t="n">
@@ -5287,7 +5440,7 @@
         </is>
       </c>
       <c r="Y49" s="3" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="Z49" s="3" t="n">
         <v>8</v>
@@ -5815,6 +5968,207 @@
       <c r="AC55" s="3" t="inlineStr">
         <is>
           <t>Polvo junto a la puerta</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="2" t="inlineStr">
+        <is>
+          <t>COM_R</t>
+        </is>
+      </c>
+      <c r="B56" s="2" t="inlineStr">
+        <is>
+          <t>COM</t>
+        </is>
+      </c>
+      <c r="C56" s="2" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="D56" s="2" t="inlineStr">
+        <is>
+          <t>COM-Pr-sin-tijera ⭐</t>
+        </is>
+      </c>
+      <c r="E56" s="2" t="inlineStr">
+        <is>
+          <t>Lugar vacío en la mesa donde el personaje cree que dejó la tijera</t>
+        </is>
+      </c>
+      <c r="F56" s="2" t="inlineStr">
+        <is>
+          <t>presente</t>
+        </is>
+      </c>
+      <c r="G56" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="H56" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="I56" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J56" s="2" t="inlineStr">
+        <is>
+          <t>sí</t>
+        </is>
+      </c>
+      <c r="K56" s="2" t="n"/>
+      <c r="L56" s="2" t="n"/>
+      <c r="M56" s="2" t="n"/>
+      <c r="N56" s="2" t="n"/>
+      <c r="O56" s="2" t="n"/>
+      <c r="P56" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q56" s="2" t="inlineStr">
+        <is>
+          <t>T_COM_R</t>
+        </is>
+      </c>
+      <c r="R56" s="2" t="n"/>
+      <c r="S56" s="2" t="n"/>
+      <c r="T56" s="2" t="n"/>
+      <c r="U56" s="2" t="n"/>
+      <c r="V56" s="2" t="n"/>
+      <c r="W56" s="2" t="n"/>
+      <c r="X56" s="2" t="inlineStr">
+        <is>
+          <t>Solo en T6 (último presente antes del primer futuro). Oculto: no se dibuja, es el punto al que camina la cinemática</t>
+        </is>
+      </c>
+      <c r="Y56" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="Z56" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="AA56" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="AB56" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="AC56" s="3" t="inlineStr">
+        <is>
+          <t>Mesa</t>
+        </is>
+      </c>
+      <c r="AD56" t="n">
+        <v>6</v>
+      </c>
+      <c r="AE56" t="inlineStr">
+        <is>
+          <t>sí</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="2" t="inlineStr">
+        <is>
+          <t>COM_S</t>
+        </is>
+      </c>
+      <c r="B57" s="2" t="inlineStr">
+        <is>
+          <t>COM</t>
+        </is>
+      </c>
+      <c r="C57" s="2" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="D57" s="2" t="inlineStr">
+        <is>
+          <t>COM-Pr-bolsillo ⭐</t>
+        </is>
+      </c>
+      <c r="E57" s="2" t="inlineStr">
+        <is>
+          <t>Diálogo obligatorio del presente: la tijera está en la mesa y en el bolsillo</t>
+        </is>
+      </c>
+      <c r="F57" s="2" t="inlineStr">
+        <is>
+          <t>presente</t>
+        </is>
+      </c>
+      <c r="G57" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="H57" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="I57" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J57" s="2" t="inlineStr">
+        <is>
+          <t>sí</t>
+        </is>
+      </c>
+      <c r="K57" s="2" t="n"/>
+      <c r="L57" s="2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="M57" s="2" t="inlineStr">
+        <is>
+          <t>COM_O.Usado</t>
+        </is>
+      </c>
+      <c r="N57" s="2" t="n"/>
+      <c r="O57" s="2" t="n"/>
+      <c r="P57" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q57" s="2" t="inlineStr">
+        <is>
+          <t>T_COM_S</t>
+        </is>
+      </c>
+      <c r="R57" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="S57" s="2" t="inlineStr">
+        <is>
+          <t>A_COM_S</t>
+        </is>
+      </c>
+      <c r="T57" s="2" t="n"/>
+      <c r="U57" s="2" t="n"/>
+      <c r="V57" s="2" t="n"/>
+      <c r="W57" s="2" t="n"/>
+      <c r="X57" s="2" t="inlineStr">
+        <is>
+          <t>Oculto (la tijera que se ve es COM_N). Obligatorio en el primer presente desde T10, salvo que se haya investigado COM_M en el pasado</t>
+        </is>
+      </c>
+      <c r="Y57" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="Z57" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="AA57" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="AB57" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="AC57" s="3" t="inlineStr">
+        <is>
+          <t>Tijera</t>
+        </is>
+      </c>
+      <c r="AE57" t="inlineStr">
+        <is>
+          <t>sí</t>
         </is>
       </c>
     </row>
@@ -6296,7 +6650,7 @@
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>presente</t>
+          <t>futuro</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
@@ -6422,12 +6776,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C4"/>
+  <dimension ref="A1:D4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
     <col width="8" customWidth="1" min="2" max="2"/>
     <col width="60" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -6446,6 +6801,11 @@
           <t>notas</t>
         </is>
       </c>
+      <c r="D1" s="4" t="inlineStr">
+        <is>
+          <t>vuelta_gratis</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
@@ -6463,6 +6823,11 @@
           <t>Pasillo corto (1 ↔ 2)</t>
         </is>
       </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>sí</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
@@ -6480,6 +6845,11 @@
           <t>Pasillo corto hacia arriba (2 ↔ 4)</t>
         </is>
       </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>sí</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
@@ -6495,6 +6865,11 @@
       <c r="C4" s="3" t="inlineStr">
         <is>
           <t>Puerta bloqueada al inicio: se abre con COM_Q (2 ↔ 3)</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>sí</t>
         </is>
       </c>
     </row>
@@ -6509,7 +6884,657 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D68"/>
+  <dimension ref="A1:I18"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="6" customWidth="1" min="3" max="3"/>
+    <col width="6" customWidth="1" min="4" max="4"/>
+    <col width="8" customWidth="1" min="5" max="5"/>
+    <col width="8" customWidth="1" min="6" max="6"/>
+    <col width="50" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>sala</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>nombre</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>y</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>ancho</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>alto</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>notas</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>solido</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>en_futuro</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>MAN</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Puesto de mando</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>7</v>
+      </c>
+      <c r="D2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E2" t="n">
+        <v>6</v>
+      </c>
+      <c r="F2" t="n">
+        <v>2</v>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>La consola de NORA y el panel eléctrico están acá</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>sí</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>COM</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Puesto de radio</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E3" t="n">
+        <v>7</v>
+      </c>
+      <c r="F3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Radio, consola y registro de transmisiones</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>sí</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>roto</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>COM</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Panel de herramientas</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>13</v>
+      </c>
+      <c r="D4" t="n">
+        <v>1</v>
+      </c>
+      <c r="E4" t="n">
+        <v>3</v>
+      </c>
+      <c r="F4" t="n">
+        <v>1</v>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>En la pared. La tijera nunca está en su hueco</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>sí</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>COM</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Mesa</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>6</v>
+      </c>
+      <c r="D5" t="n">
+        <v>6</v>
+      </c>
+      <c r="E5" t="n">
+        <v>6</v>
+      </c>
+      <c r="F5" t="n">
+        <v>2</v>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Acá aparece la tijera (10,7) y las hojas de protocolo</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>sí</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>COM</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Mesita</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>3</v>
+      </c>
+      <c r="D6" t="n">
+        <v>8</v>
+      </c>
+      <c r="E6" t="n">
+        <v>2</v>
+      </c>
+      <c r="F6" t="n">
+        <v>1</v>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Donde está la taza de café del pasado</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>sí</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>SCO</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Mesa larga</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>7</v>
+      </c>
+      <c r="D7" t="n">
+        <v>5</v>
+      </c>
+      <c r="E7" t="n">
+        <v>8</v>
+      </c>
+      <c r="F7" t="n">
+        <v>2</v>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>8 sillas alrededor (3 arriba dejando lugar frente a la taza y las cartas, 4 abajo, 1 en la cabecera). La novena es la que se vuelca (objetos SCO_H / SCO_R)</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>sí</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>roto</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>SCO</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Silla</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>8</v>
+      </c>
+      <c r="D8" t="n">
+        <v>4</v>
+      </c>
+      <c r="E8" t="n">
+        <v>1</v>
+      </c>
+      <c r="F8" t="n">
+        <v>1</v>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>sí</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>caído</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>SCO</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Silla</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>11</v>
+      </c>
+      <c r="D9" t="n">
+        <v>4</v>
+      </c>
+      <c r="E9" t="n">
+        <v>1</v>
+      </c>
+      <c r="F9" t="n">
+        <v>1</v>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>sí</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>caído</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>SCO</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Silla</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>14</v>
+      </c>
+      <c r="D10" t="n">
+        <v>4</v>
+      </c>
+      <c r="E10" t="n">
+        <v>1</v>
+      </c>
+      <c r="F10" t="n">
+        <v>1</v>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>sí</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>caído</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>SCO</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Silla</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>8</v>
+      </c>
+      <c r="D11" t="n">
+        <v>7</v>
+      </c>
+      <c r="E11" t="n">
+        <v>1</v>
+      </c>
+      <c r="F11" t="n">
+        <v>1</v>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>sí</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>caído</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>SCO</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Silla</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>10</v>
+      </c>
+      <c r="D12" t="n">
+        <v>7</v>
+      </c>
+      <c r="E12" t="n">
+        <v>1</v>
+      </c>
+      <c r="F12" t="n">
+        <v>1</v>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>sí</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>caído</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>SCO</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Silla</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>12</v>
+      </c>
+      <c r="D13" t="n">
+        <v>7</v>
+      </c>
+      <c r="E13" t="n">
+        <v>1</v>
+      </c>
+      <c r="F13" t="n">
+        <v>1</v>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>sí</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>caído</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>SCO</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Silla</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>14</v>
+      </c>
+      <c r="D14" t="n">
+        <v>7</v>
+      </c>
+      <c r="E14" t="n">
+        <v>1</v>
+      </c>
+      <c r="F14" t="n">
+        <v>1</v>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>sí</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>caído</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>SCO</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Silla</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>15</v>
+      </c>
+      <c r="D15" t="n">
+        <v>5</v>
+      </c>
+      <c r="E15" t="n">
+        <v>1</v>
+      </c>
+      <c r="F15" t="n">
+        <v>1</v>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>sí</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>caído</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>SCO</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Ganchos de tazas</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>1</v>
+      </c>
+      <c r="D16" t="n">
+        <v>1</v>
+      </c>
+      <c r="E16" t="n">
+        <v>3</v>
+      </c>
+      <c r="F16" t="n">
+        <v>1</v>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>La taza con su nombre cuelga acá</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>sí</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>SCO</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Pizarra de turnos</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>10</v>
+      </c>
+      <c r="D17" t="n">
+        <v>1</v>
+      </c>
+      <c r="E17" t="n">
+        <v>4</v>
+      </c>
+      <c r="F17" t="n">
+        <v>1</v>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>sí</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>SCO</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Dispensador de agua</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
+        <v>19</v>
+      </c>
+      <c r="D18" t="n">
+        <v>1</v>
+      </c>
+      <c r="E18" t="n">
+        <v>1</v>
+      </c>
+      <c r="F18" t="n">
+        <v>2</v>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>sí</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D77"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -7123,7 +8148,7 @@
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>T_COM_C</t>
+          <t>T_COM_D</t>
         </is>
       </c>
       <c r="B31" s="2" t="n">
@@ -7136,14 +8161,14 @@
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>Todo ordenado. Menos la tijera, que no está.</t>
+          <t>Operador de comunicaciones… es mi nombre. No recuerdo haber trabajado acá.</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>T_COM_D</t>
+          <t>T_COM_E</t>
         </is>
       </c>
       <c r="B32" s="2" t="n">
@@ -7156,14 +8181,14 @@
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>Operador de comunicaciones… es mi nombre. No recuerdo haber trabajado acá.</t>
+          <t>Solo estática. Giro el dial hasta que se estabiliza: 7.41.</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>T_COM_E</t>
+          <t>T_COM_F</t>
         </is>
       </c>
       <c r="B33" s="2" t="n">
@@ -7176,14 +8201,14 @@
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>Solo estática. Giro el dial hasta que se estabiliza: 7.41.</t>
+          <t>Un plano de evacuación. Arriba de comunicaciones no hay nada. Ni la sala de la puerta.</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>T_COM_F</t>
+          <t>T_COM_G</t>
         </is>
       </c>
       <c r="B34" s="2" t="n">
@@ -7196,14 +8221,14 @@
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>Un plano de evacuación. Arriba de comunicaciones no hay nada. Ni la sala de la puerta.</t>
+          <t>Agarro una hoja y se rompe. La dejo ahí.</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>T_COM_G</t>
+          <t>T_COM_H</t>
         </is>
       </c>
       <c r="B35" s="2" t="n">
@@ -7216,14 +8241,14 @@
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>Agarro una hoja y se rompe. La dejo ahí.</t>
+          <t>Registro de transmisiones. Todo rutinario. La última entrada: 7.41. La fecha no se lee.</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>T_COM_H</t>
+          <t>T_COM_I</t>
         </is>
       </c>
       <c r="B36" s="2" t="n">
@@ -7236,14 +8261,14 @@
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>Registro de transmisiones. Todo rutinario. La última entrada: 7.41. La fecha no se lee.</t>
+          <t>Está destrozada. Todavía chisporrotea.</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>T_COM_I</t>
+          <t>T_COM_J</t>
         </is>
       </c>
       <c r="B37" s="2" t="n">
@@ -7256,14 +8281,14 @@
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>Está destrozada. Todavía chisporrotea.</t>
+          <t>Paso el dedo por la silueta de la tijera. Siempre faltó acá.</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>T_COM_J</t>
+          <t>T_COM_K</t>
         </is>
       </c>
       <c r="B38" s="2" t="n">
@@ -7276,14 +8301,14 @@
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>Paso el dedo por la silueta de la tijera. Siempre faltó acá.</t>
+          <t>El mismo plano, amarillento. Se despega de la pared.</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>T_COM_K</t>
+          <t>T_COM_L</t>
         </is>
       </c>
       <c r="B39" s="2" t="n">
@@ -7296,14 +8321,14 @@
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>El mismo plano, amarillento. Se despega de la pared.</t>
+          <t>Una nota pegada en la radio: 7.41. Es mi letra. No recuerdo haber escrito esto.</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>T_COM_L</t>
+          <t>T_COM_O</t>
         </is>
       </c>
       <c r="B40" s="2" t="n">
@@ -7316,14 +8341,14 @@
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>Una nota pegada en la radio: 7.41. Es mi letra. No recuerdo haber escrito esto.</t>
+          <t>La tijera, llena de polvo. La guardo en el bolsillo.</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>T_COM_M</t>
+          <t>T_COM_Q</t>
         </is>
       </c>
       <c r="B41" s="2" t="n">
@@ -7336,18 +8361,18 @@
       </c>
       <c r="D41" s="2" t="inlineStr">
         <is>
-          <t>Una tijera sobre la mesa.</t>
+          <t>La puerta de la sala común cede. Adentro está todo a oscuras.</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>T_COM_M</t>
+          <t>T_SCO_A</t>
         </is>
       </c>
       <c r="B42" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
@@ -7356,14 +8381,14 @@
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>¿Esto ya estaba acá? No lo recuerdo.</t>
+          <t>Nueve sillas, todas en su lugar.</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>T_COM_O</t>
+          <t>T_SCO_B</t>
         </is>
       </c>
       <c r="B43" s="2" t="n">
@@ -7376,14 +8401,14 @@
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t>La tijera, llena de polvo. La guardo en el bolsillo.</t>
+          <t>El dispensador funciona. El agua está fría.</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>T_COM_Q</t>
+          <t>T_SCO_C</t>
         </is>
       </c>
       <c r="B44" s="2" t="n">
@@ -7396,14 +8421,14 @@
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>La puerta de la sala común cede. Adentro está todo a oscuras.</t>
+          <t>La pizarra de turnos. Nueve nombres. El mío está ahí.</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>T_SCO_A</t>
+          <t>T_SCO_D</t>
         </is>
       </c>
       <c r="B45" s="2" t="n">
@@ -7416,14 +8441,14 @@
       </c>
       <c r="D45" s="2" t="inlineStr">
         <is>
-          <t>Nueve sillas, todas en su lugar.</t>
+          <t>Una taza con mi nombre. La descuelgo y la dejo sobre la mesa.</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>T_SCO_B</t>
+          <t>T_SCO_E</t>
         </is>
       </c>
       <c r="B46" s="2" t="n">
@@ -7436,14 +8461,14 @@
       </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t>El dispensador funciona. El agua está fría.</t>
+          <t>Un calendario. Los días están tachados hasta el 112.</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>T_SCO_C</t>
+          <t>T_SCO_F</t>
         </is>
       </c>
       <c r="B47" s="2" t="n">
@@ -7456,14 +8481,14 @@
       </c>
       <c r="D47" s="2" t="inlineStr">
         <is>
-          <t>La pizarra de turnos. Nueve nombres. El mío está ahí.</t>
+          <t>Una foto de la tripulación. Nueve personas. Yo estoy ahí.</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>T_SCO_D</t>
+          <t>T_SCO_G</t>
         </is>
       </c>
       <c r="B48" s="2" t="n">
@@ -7476,14 +8501,14 @@
       </c>
       <c r="D48" s="2" t="inlineStr">
         <is>
-          <t>Una taza con mi nombre. La descuelgo y la dejo sobre la mesa.</t>
+          <t>Nueve manos repartidas. Se fueron en medio de la partida.</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
         <is>
-          <t>T_SCO_E</t>
+          <t>T_SCO_H</t>
         </is>
       </c>
       <c r="B49" s="2" t="n">
@@ -7496,14 +8521,14 @@
       </c>
       <c r="D49" s="2" t="inlineStr">
         <is>
-          <t>Un calendario. Los días están tachados hasta el 112.</t>
+          <t>Una silla volcada. La levanto.</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>T_SCO_F</t>
+          <t>T_SCO_I</t>
         </is>
       </c>
       <c r="B50" s="2" t="n">
@@ -7516,14 +8541,14 @@
       </c>
       <c r="D50" s="2" t="inlineStr">
         <is>
-          <t>Una foto de la tripulación. Nueve personas. Yo estoy ahí.</t>
+          <t>Una taza con mi nombre.</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
         <is>
-          <t>T_SCO_G</t>
+          <t>T_SCO_J</t>
         </is>
       </c>
       <c r="B51" s="2" t="n">
@@ -7536,14 +8561,14 @@
       </c>
       <c r="D51" s="2" t="inlineStr">
         <is>
-          <t>Nueve manos repartidas. Se fueron en medio de la partida.</t>
+          <t>La taza está sobre la mesa, con un resto seco de café. ¿No estaba colgada?</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>T_SCO_H</t>
+          <t>T_SCO_K</t>
         </is>
       </c>
       <c r="B52" s="2" t="n">
@@ -7556,14 +8581,14 @@
       </c>
       <c r="D52" s="2" t="inlineStr">
         <is>
-          <t>Una silla volcada. La levanto.</t>
+          <t>La pizarra de turnos, borrada a medias. Varios nombres no se leen.</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
         <is>
-          <t>T_SCO_I</t>
+          <t>T_SCO_L</t>
         </is>
       </c>
       <c r="B53" s="2" t="n">
@@ -7576,14 +8601,14 @@
       </c>
       <c r="D53" s="2" t="inlineStr">
         <is>
-          <t>Una taza con mi nombre.</t>
+          <t>El reloj está detenido: 03:12.</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>T_SCO_J</t>
+          <t>T_SCO_M</t>
         </is>
       </c>
       <c r="B54" s="2" t="n">
@@ -7596,14 +8621,14 @@
       </c>
       <c r="D54" s="2" t="inlineStr">
         <is>
-          <t>La taza está sobre la mesa, con un resto seco de café. ¿No estaba colgada?</t>
+          <t>Una chaqueta olvidada en el respaldo.</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
         <is>
-          <t>T_SCO_K</t>
+          <t>T_SCO_N</t>
         </is>
       </c>
       <c r="B55" s="2" t="n">
@@ -7616,14 +8641,14 @@
       </c>
       <c r="D55" s="2" t="inlineStr">
         <is>
-          <t>La pizarra de turnos, borrada a medias. Varios nombres no se leen.</t>
+          <t>La mesa está partida al medio.</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>T_SCO_L</t>
+          <t>T_SCO_O</t>
         </is>
       </c>
       <c r="B56" s="2" t="n">
@@ -7636,14 +8661,14 @@
       </c>
       <c r="D56" s="2" t="inlineStr">
         <is>
-          <t>El reloj está detenido: 03:12.</t>
+          <t>Mi taza. Rota.</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
         <is>
-          <t>T_SCO_M</t>
+          <t>T_SCO_P</t>
         </is>
       </c>
       <c r="B57" s="2" t="n">
@@ -7656,14 +8681,14 @@
       </c>
       <c r="D57" s="2" t="inlineStr">
         <is>
-          <t>Una chaqueta olvidada en el respaldo.</t>
+          <t>El calendario, en el piso. No se lee nada.</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>T_SCO_N</t>
+          <t>T_SCO_Q</t>
         </is>
       </c>
       <c r="B58" s="2" t="n">
@@ -7676,14 +8701,14 @@
       </c>
       <c r="D58" s="2" t="inlineStr">
         <is>
-          <t>La mesa está partida al medio.</t>
+          <t>El dispensador está seco. Cuelgan cables.</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
         <is>
-          <t>T_SCO_O</t>
+          <t>T_SCO_S</t>
         </is>
       </c>
       <c r="B59" s="2" t="n">
@@ -7696,14 +8721,14 @@
       </c>
       <c r="D59" s="2" t="inlineStr">
         <is>
-          <t>Mi taza. Rota.</t>
+          <t>No ceden. Algo las traba.</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>T_SCO_P</t>
+          <t>T_PTA_A</t>
         </is>
       </c>
       <c r="B60" s="2" t="n">
@@ -7716,34 +8741,34 @@
       </c>
       <c r="D60" s="2" t="inlineStr">
         <is>
-          <t>El calendario, en el piso. No se lee nada.</t>
+          <t>Una puerta. Está cerrada.</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
         <is>
-          <t>T_SCO_Q</t>
+          <t>T_PTA_A</t>
         </is>
       </c>
       <c r="B61" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C61" s="2" t="inlineStr">
         <is>
-          <t>PERSONAJE</t>
+          <t>NORA</t>
         </is>
       </c>
       <c r="D61" s="2" t="inlineStr">
         <is>
-          <t>El dispensador está seco. Cuelgan cables.</t>
+          <t>No tengo registros de esa puerta. Esta sala no figura en mi mapa interno.</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>T_SCO_S</t>
+          <t>T_PTA_B</t>
         </is>
       </c>
       <c r="B62" s="2" t="n">
@@ -7756,14 +8781,14 @@
       </c>
       <c r="D62" s="2" t="inlineStr">
         <is>
-          <t>No ceden. Algo las traba.</t>
+          <t>Tiene soporte. No tiene nombre.</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
         <is>
-          <t>T_PTA_A</t>
+          <t>T_PTA_C</t>
         </is>
       </c>
       <c r="B63" s="2" t="n">
@@ -7776,34 +8801,34 @@
       </c>
       <c r="D63" s="2" t="inlineStr">
         <is>
-          <t>Una puerta. Está cerrada.</t>
+          <t>Todavía tiene el plástico protector. Parece nueva.</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>T_PTA_A</t>
+          <t>T_PTA_D</t>
         </is>
       </c>
       <c r="B64" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C64" s="2" t="inlineStr">
         <is>
-          <t>NORA</t>
+          <t>PERSONAJE</t>
         </is>
       </c>
       <c r="D64" s="2" t="inlineStr">
         <is>
-          <t>No tengo registros de esa puerta. Esta sala no figura en mi mapa interno.</t>
+          <t>Oxidada. Sigue cerrada.</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
         <is>
-          <t>T_PTA_B</t>
+          <t>T_PTA_E</t>
         </is>
       </c>
       <c r="B65" s="2" t="n">
@@ -7816,14 +8841,14 @@
       </c>
       <c r="D65" s="2" t="inlineStr">
         <is>
-          <t>Tiene soporte. No tiene nombre.</t>
+          <t>Polvo acumulado contra la puerta. Nadie la tocó en mucho tiempo.</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>T_PTA_C</t>
+          <t>T_COM_C</t>
         </is>
       </c>
       <c r="B66" s="2" t="n">
@@ -7836,14 +8861,14 @@
       </c>
       <c r="D66" s="2" t="inlineStr">
         <is>
-          <t>Todavía tiene el plástico protector. Parece nueva.</t>
+          <t>Todo ordenado. Menos la tijera, que no está en su lugar.</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
         <is>
-          <t>T_PTA_D</t>
+          <t>T_COM_R</t>
         </is>
       </c>
       <c r="B67" s="2" t="n">
@@ -7856,14 +8881,14 @@
       </c>
       <c r="D67" s="2" t="inlineStr">
         <is>
-          <t>Oxidada. Sigue cerrada.</t>
+          <t>Pensé que había dejado la tijera acá.</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>T_PTA_E</t>
+          <t>SIS_SIN_ENERGIA</t>
         </is>
       </c>
       <c r="B68" s="2" t="n">
@@ -7876,7 +8901,187 @@
       </c>
       <c r="D68" s="2" t="inlineStr">
         <is>
-          <t>Polvo acumulado contra la puerta. Nadie la tocó en mucho tiempo.</t>
+          <t>Me quedé sin energía. Tengo que volver.</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="2" t="inlineStr">
+        <is>
+          <t>SIS_DESCANSAR_PREGUNTA</t>
+        </is>
+      </c>
+      <c r="B69" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C69" s="2" t="inlineStr">
+        <is>
+          <t>NORA</t>
+        </is>
+      </c>
+      <c r="D69" s="2" t="inlineStr">
+        <is>
+          <t>No tengo nada nuevo para informarle. ¿Desea descansar?</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="2" t="inlineStr">
+        <is>
+          <t>SIS_DESCANSAR_SI</t>
+        </is>
+      </c>
+      <c r="B70" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C70" s="2" t="inlineStr">
+        <is>
+          <t>PERSONAJE</t>
+        </is>
+      </c>
+      <c r="D70" s="2" t="inlineStr">
+        <is>
+          <t>Voy a descansar un rato.</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="2" t="inlineStr">
+        <is>
+          <t>T_COM_M</t>
+        </is>
+      </c>
+      <c r="B71" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C71" s="2" t="inlineStr">
+        <is>
+          <t>PERSONAJE</t>
+        </is>
+      </c>
+      <c r="D71" s="2" t="inlineStr">
+        <is>
+          <t>¿La tijera?</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="2" t="inlineStr">
+        <is>
+          <t>T_COM_M</t>
+        </is>
+      </c>
+      <c r="B72" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="C72" s="2" t="inlineStr">
+        <is>
+          <t>PERSONAJE</t>
+        </is>
+      </c>
+      <c r="D72" s="2" t="inlineStr">
+        <is>
+          <t>¿Cómo puede estar acá, si la acabo de agarrar?</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="2" t="inlineStr">
+        <is>
+          <t>T_COM_M</t>
+        </is>
+      </c>
+      <c r="B73" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="C73" s="2" t="inlineStr">
+        <is>
+          <t>PERSONAJE</t>
+        </is>
+      </c>
+      <c r="D73" s="2" t="inlineStr">
+        <is>
+          <t>Me toco el bolsillo. La tengo acá. Hay dos.</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="2" t="inlineStr">
+        <is>
+          <t>T_COM_S</t>
+        </is>
+      </c>
+      <c r="B74" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C74" s="2" t="inlineStr">
+        <is>
+          <t>PERSONAJE</t>
+        </is>
+      </c>
+      <c r="D74" s="2" t="inlineStr">
+        <is>
+          <t>Qué raro… acá está la tijera.</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="2" t="inlineStr">
+        <is>
+          <t>T_COM_S</t>
+        </is>
+      </c>
+      <c r="B75" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="C75" s="2" t="inlineStr">
+        <is>
+          <t>PERSONAJE</t>
+        </is>
+      </c>
+      <c r="D75" s="2" t="inlineStr">
+        <is>
+          <t>Pero si yo la había agarrado.</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="2" t="inlineStr">
+        <is>
+          <t>T_COM_S</t>
+        </is>
+      </c>
+      <c r="B76" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="C76" s="2" t="inlineStr">
+        <is>
+          <t>PERSONAJE</t>
+        </is>
+      </c>
+      <c r="D76" s="2" t="inlineStr">
+        <is>
+          <t>Me toco el bolsillo. Está acá.</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="2" t="inlineStr">
+        <is>
+          <t>T_COM_S</t>
+        </is>
+      </c>
+      <c r="B77" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="C77" s="2" t="inlineStr">
+        <is>
+          <t>PERSONAJE</t>
+        </is>
+      </c>
+      <c r="D77" s="2" t="inlineStr">
+        <is>
+          <t>¿Cómo puede ser?</t>
         </is>
       </c>
     </row>
@@ -7886,13 +9091,13 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B21"/>
+  <dimension ref="A1:B23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -8151,13 +9356,37 @@
         </is>
       </c>
     </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>A_COM_M</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>Hay una tijera en la mesa de comunicaciones, aunque la mía la tengo en el bolsillo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>A_COM_S</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>La tijera está sobre la mesa de comunicaciones. Y también en mi bolsillo.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:B21"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -8209,59 +9438,4 @@
   <autoFilter ref="A1:C2"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:B3"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="16" customWidth="1" min="1" max="1"/>
-    <col width="60" customWidth="1" min="2" max="2"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>id</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>descripcion</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>estatica</t>
-        </is>
-      </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>Estática de radio (placeholder)</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>chisporroteo</t>
-        </is>
-      </c>
-      <c r="B3" s="2" t="inlineStr">
-        <is>
-          <t>Chisporroteo eléctrico (placeholder)</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <autoFilter ref="A1:B3"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
Paso 8: NORA, anotaciones e inventario
</commit_message>
<xml_diff>
--- a/planilla/contenido_alfa.xlsx
+++ b/planilla/contenido_alfa.xlsx
@@ -7534,7 +7534,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D77"/>
+  <dimension ref="A1:D78"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -8948,7 +8948,7 @@
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
         <is>
-          <t>T_COM_M</t>
+          <t>SIS_NORA_MENU</t>
         </is>
       </c>
       <c r="B71" s="2" t="n">
@@ -8956,12 +8956,12 @@
       </c>
       <c r="C71" s="2" t="inlineStr">
         <is>
-          <t>PERSONAJE</t>
+          <t>NORA</t>
         </is>
       </c>
       <c r="D71" s="2" t="inlineStr">
         <is>
-          <t>¿La tijera?</t>
+          <t>¿En qué puedo ayudarle?</t>
         </is>
       </c>
     </row>
@@ -8972,7 +8972,7 @@
         </is>
       </c>
       <c r="B72" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C72" s="2" t="inlineStr">
         <is>
@@ -8981,7 +8981,7 @@
       </c>
       <c r="D72" s="2" t="inlineStr">
         <is>
-          <t>¿Cómo puede estar acá, si la acabo de agarrar?</t>
+          <t>¿La tijera?</t>
         </is>
       </c>
     </row>
@@ -8992,7 +8992,7 @@
         </is>
       </c>
       <c r="B73" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C73" s="2" t="inlineStr">
         <is>
@@ -9001,18 +9001,18 @@
       </c>
       <c r="D73" s="2" t="inlineStr">
         <is>
-          <t>Me toco el bolsillo. La tengo acá. Hay dos.</t>
+          <t>¿Cómo puede estar acá, si la acabo de agarrar?</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
         <is>
-          <t>T_COM_S</t>
+          <t>T_COM_M</t>
         </is>
       </c>
       <c r="B74" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C74" s="2" t="inlineStr">
         <is>
@@ -9021,7 +9021,7 @@
       </c>
       <c r="D74" s="2" t="inlineStr">
         <is>
-          <t>Qué raro… acá está la tijera.</t>
+          <t>Me toco el bolsillo. La tengo acá. Hay dos.</t>
         </is>
       </c>
     </row>
@@ -9032,7 +9032,7 @@
         </is>
       </c>
       <c r="B75" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C75" s="2" t="inlineStr">
         <is>
@@ -9041,7 +9041,7 @@
       </c>
       <c r="D75" s="2" t="inlineStr">
         <is>
-          <t>Pero si yo la había agarrado.</t>
+          <t>Qué raro… acá está la tijera.</t>
         </is>
       </c>
     </row>
@@ -9052,7 +9052,7 @@
         </is>
       </c>
       <c r="B76" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C76" s="2" t="inlineStr">
         <is>
@@ -9061,7 +9061,7 @@
       </c>
       <c r="D76" s="2" t="inlineStr">
         <is>
-          <t>Me toco el bolsillo. Está acá.</t>
+          <t>Pero si yo la había agarrado.</t>
         </is>
       </c>
     </row>
@@ -9072,14 +9072,34 @@
         </is>
       </c>
       <c r="B77" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="C77" s="2" t="inlineStr">
+        <is>
+          <t>PERSONAJE</t>
+        </is>
+      </c>
+      <c r="D77" s="2" t="inlineStr">
+        <is>
+          <t>Me toco el bolsillo. Está acá.</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="2" t="inlineStr">
+        <is>
+          <t>T_COM_S</t>
+        </is>
+      </c>
+      <c r="B78" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="C77" s="2" t="inlineStr">
+      <c r="C78" s="2" t="inlineStr">
         <is>
           <t>PERSONAJE</t>
         </is>
       </c>
-      <c r="D77" s="2" t="inlineStr">
+      <c r="D78" s="2" t="inlineStr">
         <is>
           <t>¿Cómo puede ser?</t>
         </is>

</xml_diff>

<commit_message>
Objetos en los 3 tiempos y sprites
</commit_message>
<xml_diff>
--- a/planilla/contenido_alfa.xlsx
+++ b/planilla/contenido_alfa.xlsx
@@ -19,6 +19,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="audios" sheetId="10" state="visible" r:id="rId10"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="eventos" sheetId="11" state="visible" r:id="rId11"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="config" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="sprites" sheetId="13" state="visible" r:id="rId13"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'LEEME'!$A$1:$A$17</definedName>
@@ -457,7 +458,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A33"/>
+  <dimension ref="A1:A36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="140" customWidth="1" min="1" max="1"/>
@@ -595,7 +596,6 @@
         </is>
       </c>
     </row>
-    <row r="21"/>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
@@ -677,6 +677,27 @@
       <c r="A33" t="inlineStr">
         <is>
           <t>La sala de mando arranca con luz máxima 2; el arreglo (evento arreglo_panel) habilita luz 3 en mando y comunicaciones y suma energia_por_arreglo (14 → 15).</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Regla de los 3 tiempos (22/10/2026): todo objeto suelto existe en pasado, presente y futuro, en el mismo lugar; las variantes sin nada nuevo son solo visuales (sin disparadores). Si falta, la ausencia es un objeto.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Sprites: hoja 'sprites' = catálogo (nombre → recorte en píxeles de una hoja de arte: cosas, cosas2, pantallas, puerta). En objetos (sprite, sprite_usado) y muebles (sprite, sprite_futuro) se escribe el nombre, opcionalmente con: girado (90°), espejo, repetir (llena el ancho), doble (dos, el segundo espejado), pared (apoyado en la pared de arriba).</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>sprite vacío = cuadro de color (greybox, cuando no hay sprite: taza, pinza, foto…). 'ninguno' = no se dibuja (lo muestra el mueble de abajo). sprite_usado = cómo se ve después de usarlo (la silla levantada, el panel arreglado).</t>
         </is>
       </c>
     </row>
@@ -977,13 +998,1081 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G43"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="20" customWidth="1" min="1" max="1"/>
+    <col width="11" customWidth="1" min="2" max="2"/>
+    <col width="6" customWidth="1" min="3" max="3"/>
+    <col width="6" customWidth="1" min="4" max="4"/>
+    <col width="7" customWidth="1" min="5" max="5"/>
+    <col width="6" customWidth="1" min="6" max="6"/>
+    <col width="40" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>nombre</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>hoja</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>y</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>ancho</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>alto</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>notas</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>consola_larga</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>cosas2</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>67</v>
+      </c>
+      <c r="D2" t="n">
+        <v>19</v>
+      </c>
+      <c r="E2" t="n">
+        <v>298</v>
+      </c>
+      <c r="F2" t="n">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>consola_naranja</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>cosas2</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>76</v>
+      </c>
+      <c r="D3" t="n">
+        <v>137</v>
+      </c>
+      <c r="E3" t="n">
+        <v>240</v>
+      </c>
+      <c r="F3" t="n">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>consola_control</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>cosas2</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>168</v>
+      </c>
+      <c r="D4" t="n">
+        <v>259</v>
+      </c>
+      <c r="E4" t="n">
+        <v>100</v>
+      </c>
+      <c r="F4" t="n">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>mesa_oscura</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>cosas2</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>72</v>
+      </c>
+      <c r="D5" t="n">
+        <v>483</v>
+      </c>
+      <c r="E5" t="n">
+        <v>146</v>
+      </c>
+      <c r="F5" t="n">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>mesa_naranja</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>cosas2</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>72</v>
+      </c>
+      <c r="D6" t="n">
+        <v>584</v>
+      </c>
+      <c r="E6" t="n">
+        <v>147</v>
+      </c>
+      <c r="F6" t="n">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>mesa_clara</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>cosas2</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>72</v>
+      </c>
+      <c r="D7" t="n">
+        <v>687</v>
+      </c>
+      <c r="E7" t="n">
+        <v>147</v>
+      </c>
+      <c r="F7" t="n">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>mesa_azul</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>cosas2</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>72</v>
+      </c>
+      <c r="D8" t="n">
+        <v>780</v>
+      </c>
+      <c r="E8" t="n">
+        <v>147</v>
+      </c>
+      <c r="F8" t="n">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>silla_frente</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>cosas2</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>295</v>
+      </c>
+      <c r="D9" t="n">
+        <v>495</v>
+      </c>
+      <c r="E9" t="n">
+        <v>33</v>
+      </c>
+      <c r="F9" t="n">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>silla_espalda</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>cosas2</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>248</v>
+      </c>
+      <c r="D10" t="n">
+        <v>576</v>
+      </c>
+      <c r="E10" t="n">
+        <v>32</v>
+      </c>
+      <c r="F10" t="n">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>silla_lado</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>cosas2</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>298</v>
+      </c>
+      <c r="D11" t="n">
+        <v>600</v>
+      </c>
+      <c r="E11" t="n">
+        <v>27</v>
+      </c>
+      <c r="F11" t="n">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>estantes</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>cosas</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>432</v>
+      </c>
+      <c r="D12" t="n">
+        <v>0</v>
+      </c>
+      <c r="E12" t="n">
+        <v>144</v>
+      </c>
+      <c r="F12" t="n">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>estante_colgado</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>cosas</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>528</v>
+      </c>
+      <c r="D13" t="n">
+        <v>0</v>
+      </c>
+      <c r="E13" t="n">
+        <v>144</v>
+      </c>
+      <c r="F13" t="n">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>hoja_a</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>cosas</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>446</v>
+      </c>
+      <c r="D14" t="n">
+        <v>159</v>
+      </c>
+      <c r="E14" t="n">
+        <v>19</v>
+      </c>
+      <c r="F14" t="n">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>hoja_b</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>cosas</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>496</v>
+      </c>
+      <c r="D15" t="n">
+        <v>161</v>
+      </c>
+      <c r="E15" t="n">
+        <v>16</v>
+      </c>
+      <c r="F15" t="n">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>hoja_c</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>cosas</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>544</v>
+      </c>
+      <c r="D16" t="n">
+        <v>158</v>
+      </c>
+      <c r="E16" t="n">
+        <v>16</v>
+      </c>
+      <c r="F16" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>hoja_suelta</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>cosas</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>447</v>
+      </c>
+      <c r="D17" t="n">
+        <v>208</v>
+      </c>
+      <c r="E17" t="n">
+        <v>18</v>
+      </c>
+      <c r="F17" t="n">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>hojas_pila</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>cosas</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
+        <v>530</v>
+      </c>
+      <c r="D18" t="n">
+        <v>196</v>
+      </c>
+      <c r="E18" t="n">
+        <v>43</v>
+      </c>
+      <c r="F18" t="n">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>hojas_rotas</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>cosas</t>
+        </is>
+      </c>
+      <c r="C19" t="n">
+        <v>673</v>
+      </c>
+      <c r="D19" t="n">
+        <v>145</v>
+      </c>
+      <c r="E19" t="n">
+        <v>45</v>
+      </c>
+      <c r="F19" t="n">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>caja_carton</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>cosas</t>
+        </is>
+      </c>
+      <c r="C20" t="n">
+        <v>640</v>
+      </c>
+      <c r="D20" t="n">
+        <v>159</v>
+      </c>
+      <c r="E20" t="n">
+        <v>16</v>
+      </c>
+      <c r="F20" t="n">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>maquina_a</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>cosas</t>
+        </is>
+      </c>
+      <c r="C21" t="n">
+        <v>638</v>
+      </c>
+      <c r="D21" t="n">
+        <v>240</v>
+      </c>
+      <c r="E21" t="n">
+        <v>35</v>
+      </c>
+      <c r="F21" t="n">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>maquina_b</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>cosas</t>
+        </is>
+      </c>
+      <c r="C22" t="n">
+        <v>672</v>
+      </c>
+      <c r="D22" t="n">
+        <v>240</v>
+      </c>
+      <c r="E22" t="n">
+        <v>25</v>
+      </c>
+      <c r="F22" t="n">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>terminal_naranja</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>cosas</t>
+        </is>
+      </c>
+      <c r="C23" t="n">
+        <v>213</v>
+      </c>
+      <c r="D23" t="n">
+        <v>355</v>
+      </c>
+      <c r="E23" t="n">
+        <v>11</v>
+      </c>
+      <c r="F23" t="n">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>terminal_azul</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>cosas</t>
+        </is>
+      </c>
+      <c r="C24" t="n">
+        <v>354</v>
+      </c>
+      <c r="D24" t="n">
+        <v>346</v>
+      </c>
+      <c r="E24" t="n">
+        <v>12</v>
+      </c>
+      <c r="F24" t="n">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>terminal_azul_b</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>cosas</t>
+        </is>
+      </c>
+      <c r="C25" t="n">
+        <v>257</v>
+      </c>
+      <c r="D25" t="n">
+        <v>432</v>
+      </c>
+      <c r="E25" t="n">
+        <v>13</v>
+      </c>
+      <c r="F25" t="n">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>terminal_naranja_b</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>cosas</t>
+        </is>
+      </c>
+      <c r="C26" t="n">
+        <v>210</v>
+      </c>
+      <c r="D26" t="n">
+        <v>490</v>
+      </c>
+      <c r="E26" t="n">
+        <v>12</v>
+      </c>
+      <c r="F26" t="n">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>terminal_cian</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>cosas</t>
+        </is>
+      </c>
+      <c r="C27" t="n">
+        <v>288</v>
+      </c>
+      <c r="D27" t="n">
+        <v>528</v>
+      </c>
+      <c r="E27" t="n">
+        <v>48</v>
+      </c>
+      <c r="F27" t="n">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>terminal_apagada</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>cosas</t>
+        </is>
+      </c>
+      <c r="C28" t="n">
+        <v>336</v>
+      </c>
+      <c r="D28" t="n">
+        <v>528</v>
+      </c>
+      <c r="E28" t="n">
+        <v>48</v>
+      </c>
+      <c r="F28" t="n">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>rejilla_luz</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>cosas</t>
+        </is>
+      </c>
+      <c r="C29" t="n">
+        <v>63</v>
+      </c>
+      <c r="D29" t="n">
+        <v>408</v>
+      </c>
+      <c r="E29" t="n">
+        <v>50</v>
+      </c>
+      <c r="F29" t="n">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>rejilla_oscura</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>cosas</t>
+        </is>
+      </c>
+      <c r="C30" t="n">
+        <v>96</v>
+      </c>
+      <c r="D30" t="n">
+        <v>498</v>
+      </c>
+      <c r="E30" t="n">
+        <v>48</v>
+      </c>
+      <c r="F30" t="n">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>cajitas</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>cosas</t>
+        </is>
+      </c>
+      <c r="C31" t="n">
+        <v>288</v>
+      </c>
+      <c r="D31" t="n">
+        <v>104</v>
+      </c>
+      <c r="E31" t="n">
+        <v>47</v>
+      </c>
+      <c r="F31" t="n">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>tacho</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>cosas</t>
+        </is>
+      </c>
+      <c r="C32" t="n">
+        <v>391</v>
+      </c>
+      <c r="D32" t="n">
+        <v>391</v>
+      </c>
+      <c r="E32" t="n">
+        <v>33</v>
+      </c>
+      <c r="F32" t="n">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>mon_azul</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>pantallas</t>
+        </is>
+      </c>
+      <c r="C33" t="n">
+        <v>1</v>
+      </c>
+      <c r="D33" t="n">
+        <v>1</v>
+      </c>
+      <c r="E33" t="n">
+        <v>46</v>
+      </c>
+      <c r="F33" t="n">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>mon_verde</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>pantallas</t>
+        </is>
+      </c>
+      <c r="C34" t="n">
+        <v>1</v>
+      </c>
+      <c r="D34" t="n">
+        <v>98</v>
+      </c>
+      <c r="E34" t="n">
+        <v>45</v>
+      </c>
+      <c r="F34" t="n">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>mon_naranja</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>pantallas</t>
+        </is>
+      </c>
+      <c r="C35" t="n">
+        <v>1</v>
+      </c>
+      <c r="D35" t="n">
+        <v>194</v>
+      </c>
+      <c r="E35" t="n">
+        <v>46</v>
+      </c>
+      <c r="F35" t="n">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>mon_rota</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>pantallas</t>
+        </is>
+      </c>
+      <c r="C36" t="n">
+        <v>2</v>
+      </c>
+      <c r="D36" t="n">
+        <v>386</v>
+      </c>
+      <c r="E36" t="n">
+        <v>44</v>
+      </c>
+      <c r="F36" t="n">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>mon_apagada</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>pantallas</t>
+        </is>
+      </c>
+      <c r="C37" t="n">
+        <v>1</v>
+      </c>
+      <c r="D37" t="n">
+        <v>482</v>
+      </c>
+      <c r="E37" t="n">
+        <v>45</v>
+      </c>
+      <c r="F37" t="n">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>panel_datos</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>pantallas</t>
+        </is>
+      </c>
+      <c r="C38" t="n">
+        <v>384</v>
+      </c>
+      <c r="D38" t="n">
+        <v>3</v>
+      </c>
+      <c r="E38" t="n">
+        <v>96</v>
+      </c>
+      <c r="F38" t="n">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>panel_cian</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>pantallas</t>
+        </is>
+      </c>
+      <c r="C39" t="n">
+        <v>384</v>
+      </c>
+      <c r="D39" t="n">
+        <v>98</v>
+      </c>
+      <c r="E39" t="n">
+        <v>96</v>
+      </c>
+      <c r="F39" t="n">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>panel_apagado</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>pantallas</t>
+        </is>
+      </c>
+      <c r="C40" t="n">
+        <v>384</v>
+      </c>
+      <c r="D40" t="n">
+        <v>291</v>
+      </c>
+      <c r="E40" t="n">
+        <v>96</v>
+      </c>
+      <c r="F40" t="n">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>panel_roto</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>pantallas</t>
+        </is>
+      </c>
+      <c r="C41" t="n">
+        <v>384</v>
+      </c>
+      <c r="D41" t="n">
+        <v>386</v>
+      </c>
+      <c r="E41" t="n">
+        <v>96</v>
+      </c>
+      <c r="F41" t="n">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>puerta</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>puerta</t>
+        </is>
+      </c>
+      <c r="C42" t="n">
+        <v>0</v>
+      </c>
+      <c r="D42" t="n">
+        <v>22</v>
+      </c>
+      <c r="E42" t="n">
+        <v>48</v>
+      </c>
+      <c r="F42" t="n">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>botella_caida</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>cosas</t>
+        </is>
+      </c>
+      <c r="C43" t="n">
+        <v>730</v>
+      </c>
+      <c r="D43" t="n">
+        <v>300</v>
+      </c>
+      <c r="E43" t="n">
+        <v>28</v>
+      </c>
+      <c r="F43" t="n">
+        <v>23</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE62"/>
+  <dimension ref="A1:AG84"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1175,6 +2264,16 @@
           <t>oculto</t>
         </is>
       </c>
+      <c r="AF1" t="inlineStr">
+        <is>
+          <t>sprite</t>
+        </is>
+      </c>
+      <c r="AG1" t="inlineStr">
+        <is>
+          <t>sprite_usado</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -1274,6 +2373,11 @@
       <c r="AC2" s="3" t="inlineStr">
         <is>
           <t>Panel eléctrico</t>
+        </is>
+      </c>
+      <c r="AF2" t="inlineStr">
+        <is>
+          <t>rejilla_oscura</t>
         </is>
       </c>
     </row>
@@ -1359,6 +2463,11 @@
           <t>Consola de NORA</t>
         </is>
       </c>
+      <c r="AF3" t="inlineStr">
+        <is>
+          <t>consola_control</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -1454,6 +2563,11 @@
           <t>Consola de NORA</t>
         </is>
       </c>
+      <c r="AF4" t="inlineStr">
+        <is>
+          <t>consola_control</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -1549,6 +2663,11 @@
           <t>Consola de NORA</t>
         </is>
       </c>
+      <c r="AF5" t="inlineStr">
+        <is>
+          <t>consola_control</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -1642,6 +2761,11 @@
       <c r="AC6" s="3" t="inlineStr">
         <is>
           <t>Consola de NORA</t>
+        </is>
+      </c>
+      <c r="AF6" t="inlineStr">
+        <is>
+          <t>consola_control</t>
         </is>
       </c>
     </row>
@@ -1735,6 +2859,11 @@
           <t>Consola de NORA</t>
         </is>
       </c>
+      <c r="AF7" t="inlineStr">
+        <is>
+          <t>consola_control</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -1826,6 +2955,11 @@
           <t>Consola de NORA</t>
         </is>
       </c>
+      <c r="AF8" t="inlineStr">
+        <is>
+          <t>consola_control</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -1917,6 +3051,11 @@
           <t>Consola de NORA</t>
         </is>
       </c>
+      <c r="AF9" t="inlineStr">
+        <is>
+          <t>consola_control</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -2008,6 +3147,11 @@
           <t>Consola de NORA</t>
         </is>
       </c>
+      <c r="AF10" t="inlineStr">
+        <is>
+          <t>consola_control</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -2105,6 +3249,11 @@
       <c r="AC11" s="3" t="inlineStr">
         <is>
           <t>Consola de NORA</t>
+        </is>
+      </c>
+      <c r="AF11" t="inlineStr">
+        <is>
+          <t>consola_control</t>
         </is>
       </c>
     </row>
@@ -2190,6 +3339,11 @@
           <t>Consola de NORA</t>
         </is>
       </c>
+      <c r="AF12" t="inlineStr">
+        <is>
+          <t>consola_control</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -2281,6 +3435,11 @@
           <t>Consola de NORA</t>
         </is>
       </c>
+      <c r="AF13" t="inlineStr">
+        <is>
+          <t>consola_control</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -2372,6 +3531,11 @@
           <t>Consola de NORA</t>
         </is>
       </c>
+      <c r="AF14" t="inlineStr">
+        <is>
+          <t>consola_control</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -2544,6 +3708,11 @@
           <t>Consola de radio</t>
         </is>
       </c>
+      <c r="AF16" t="inlineStr">
+        <is>
+          <t>mon_naranja</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -2633,6 +3802,11 @@
           <t>Panel de herramientas</t>
         </is>
       </c>
+      <c r="AF17" t="inlineStr">
+        <is>
+          <t>ninguno</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -2722,6 +3896,11 @@
           <t>Lista de turnos</t>
         </is>
       </c>
+      <c r="AF18" t="inlineStr">
+        <is>
+          <t>terminal_azul</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -2815,6 +3994,11 @@
       <c r="AC19" s="3" t="inlineStr">
         <is>
           <t>Radio</t>
+        </is>
+      </c>
+      <c r="AF19" t="inlineStr">
+        <is>
+          <t>mon_azul</t>
         </is>
       </c>
     </row>
@@ -2904,6 +4088,11 @@
       <c r="AC20" s="3" t="inlineStr">
         <is>
           <t>Plano de evacuación</t>
+        </is>
+      </c>
+      <c r="AF20" t="inlineStr">
+        <is>
+          <t>terminal_naranja</t>
         </is>
       </c>
     </row>
@@ -2989,6 +4178,11 @@
           <t>Hojas de protocolo</t>
         </is>
       </c>
+      <c r="AF21" t="inlineStr">
+        <is>
+          <t>hojas_pila</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -3078,6 +4272,11 @@
           <t>Registro de transmisiones</t>
         </is>
       </c>
+      <c r="AF22" t="inlineStr">
+        <is>
+          <t>terminal_cian</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -3165,6 +4364,11 @@
       <c r="AC23" s="3" t="inlineStr">
         <is>
           <t>Consola de radio</t>
+        </is>
+      </c>
+      <c r="AF23" t="inlineStr">
+        <is>
+          <t>mon_rota</t>
         </is>
       </c>
     </row>
@@ -3252,6 +4456,11 @@
       <c r="AC24" s="3" t="inlineStr">
         <is>
           <t>Panel de herramientas</t>
+        </is>
+      </c>
+      <c r="AF24" t="inlineStr">
+        <is>
+          <t>ninguno</t>
         </is>
       </c>
     </row>
@@ -3337,6 +4546,11 @@
           <t>Plano de evacuación</t>
         </is>
       </c>
+      <c r="AF25" t="inlineStr">
+        <is>
+          <t>terminal_naranja_b</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -3436,6 +4650,11 @@
       <c r="AC26" s="3" t="inlineStr">
         <is>
           <t>Nota en la radio</t>
+        </is>
+      </c>
+      <c r="AF26" t="inlineStr">
+        <is>
+          <t>hoja_suelta</t>
         </is>
       </c>
     </row>
@@ -3828,6 +5047,11 @@
           <t>Hoja rota</t>
         </is>
       </c>
+      <c r="AF30" t="inlineStr">
+        <is>
+          <t>hojas_rotas</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -3919,6 +5143,11 @@
       <c r="AC31" s="3" t="inlineStr">
         <is>
           <t>Puerta de la sala común</t>
+        </is>
+      </c>
+      <c r="AF31" t="inlineStr">
+        <is>
+          <t>ninguno</t>
         </is>
       </c>
     </row>
@@ -4008,6 +5237,11 @@
       <c r="AC32" s="3" t="inlineStr">
         <is>
           <t>Mesa larga</t>
+        </is>
+      </c>
+      <c r="AF32" t="inlineStr">
+        <is>
+          <t>ninguno</t>
         </is>
       </c>
     </row>
@@ -4093,6 +5327,11 @@
           <t>Dispensador de agua</t>
         </is>
       </c>
+      <c r="AF33" t="inlineStr">
+        <is>
+          <t>maquina_b</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -4182,6 +5421,11 @@
           <t>Pizarra de turnos</t>
         </is>
       </c>
+      <c r="AF34" t="inlineStr">
+        <is>
+          <t>panel_cian</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
@@ -4311,7 +5555,7 @@
         <v>1</v>
       </c>
       <c r="H36" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I36" s="2" t="n">
         <v>4</v>
@@ -4368,6 +5612,11 @@
           <t>Calendario</t>
         </is>
       </c>
+      <c r="AF36" t="inlineStr">
+        <is>
+          <t>hoja_c</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -4404,7 +5653,7 @@
         <v>1</v>
       </c>
       <c r="H37" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I37" s="2" t="n">
         <v>4</v>
@@ -4631,6 +5880,16 @@
       <c r="AC39" s="3" t="inlineStr">
         <is>
           <t>Silla volcada</t>
+        </is>
+      </c>
+      <c r="AF39" t="inlineStr">
+        <is>
+          <t>silla_frente girado</t>
+        </is>
+      </c>
+      <c r="AG39" t="inlineStr">
+        <is>
+          <t>silla_frente</t>
         </is>
       </c>
     </row>
@@ -4902,6 +6161,11 @@
           <t>Pizarra de turnos</t>
         </is>
       </c>
+      <c r="AF42" t="inlineStr">
+        <is>
+          <t>panel_datos</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
@@ -4938,7 +6202,7 @@
         <v>1</v>
       </c>
       <c r="H43" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I43" s="2" t="n">
         <v>4</v>
@@ -5031,7 +6295,7 @@
         <v>1</v>
       </c>
       <c r="H44" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I44" s="2" t="n">
         <v>4</v>
@@ -5165,6 +6429,11 @@
           <t>Mesa partida</t>
         </is>
       </c>
+      <c r="AF45" t="inlineStr">
+        <is>
+          <t>ninguno</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
@@ -5298,7 +6567,7 @@
         <v>1</v>
       </c>
       <c r="H47" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I47" s="2" t="n">
         <v>4</v>
@@ -5349,6 +6618,11 @@
           <t>Calendario caído</t>
         </is>
       </c>
+      <c r="AF47" t="inlineStr">
+        <is>
+          <t>hoja_suelta</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
@@ -5385,7 +6659,7 @@
         <v>1</v>
       </c>
       <c r="H48" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I48" s="2" t="n">
         <v>4</v>
@@ -5434,6 +6708,11 @@
       <c r="AC48" s="3" t="inlineStr">
         <is>
           <t>Dispensador de agua</t>
+        </is>
+      </c>
+      <c r="AF48" t="inlineStr">
+        <is>
+          <t>maquina_b</t>
         </is>
       </c>
     </row>
@@ -5525,6 +6804,11 @@
           <t>Silla</t>
         </is>
       </c>
+      <c r="AF49" t="inlineStr">
+        <is>
+          <t>silla_frente</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
@@ -5699,6 +6983,11 @@
       <c r="AC51" s="3" t="inlineStr">
         <is>
           <t>Puerta</t>
+        </is>
+      </c>
+      <c r="AF51" t="inlineStr">
+        <is>
+          <t>puerta doble pared</t>
         </is>
       </c>
     </row>
@@ -5873,6 +7162,11 @@
           <t>Puerta</t>
         </is>
       </c>
+      <c r="AF53" t="inlineStr">
+        <is>
+          <t>puerta doble pared</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
@@ -5956,6 +7250,11 @@
           <t>Puerta</t>
         </is>
       </c>
+      <c r="AF54" t="inlineStr">
+        <is>
+          <t>puerta doble pared</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
@@ -6326,6 +7625,11 @@
           <t>Consola de NORA</t>
         </is>
       </c>
+      <c r="AF58" t="inlineStr">
+        <is>
+          <t>consola_control</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -6405,6 +7709,11 @@
       <c r="AD59" t="n">
         <v>2</v>
       </c>
+      <c r="AF59" t="inlineStr">
+        <is>
+          <t>consola_control</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -6627,6 +7936,16 @@
           <t>Panel eléctrico</t>
         </is>
       </c>
+      <c r="AF61" t="inlineStr">
+        <is>
+          <t>rejilla_oscura</t>
+        </is>
+      </c>
+      <c r="AG61" t="inlineStr">
+        <is>
+          <t>rejilla_luz</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -6721,20 +8040,1582 @@
         </is>
       </c>
       <c r="Y62" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="Z62" t="n">
         <v>1</v>
       </c>
       <c r="AA62" t="n">
+        <v>1</v>
+      </c>
+      <c r="AB62" t="n">
+        <v>1</v>
+      </c>
+      <c r="AC62" t="inlineStr">
+        <is>
+          <t>Destornillador</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>COM_V</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>COM</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>variante (regla de los 3 tiempos)</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>Taza de café fría, con un borde de café seco</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>presente</t>
+        </is>
+      </c>
+      <c r="G63" t="n">
+        <v>1</v>
+      </c>
+      <c r="H63" t="n">
+        <v>1</v>
+      </c>
+      <c r="I63" t="n">
+        <v>0</v>
+      </c>
+      <c r="J63" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="X63" t="inlineStr">
+        <is>
+          <t>Solo visual: la misma cosa en otro tiempo</t>
+        </is>
+      </c>
+      <c r="Y63" t="n">
+        <v>4</v>
+      </c>
+      <c r="Z63" t="n">
+        <v>8</v>
+      </c>
+      <c r="AA63" t="n">
+        <v>1</v>
+      </c>
+      <c r="AB63" t="n">
+        <v>1</v>
+      </c>
+      <c r="AC63" t="inlineStr">
+        <is>
+          <t>Taza de café</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>COM_W</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>COM</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>variante (regla de los 3 tiempos)</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>Taza de café rota sobre la mesita</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>futuro</t>
+        </is>
+      </c>
+      <c r="G64" t="n">
+        <v>1</v>
+      </c>
+      <c r="H64" t="n">
+        <v>1</v>
+      </c>
+      <c r="I64" t="n">
+        <v>0</v>
+      </c>
+      <c r="J64" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="X64" t="inlineStr">
+        <is>
+          <t>Solo visual: la misma cosa en otro tiempo</t>
+        </is>
+      </c>
+      <c r="Y64" t="n">
+        <v>4</v>
+      </c>
+      <c r="Z64" t="n">
+        <v>8</v>
+      </c>
+      <c r="AA64" t="n">
+        <v>1</v>
+      </c>
+      <c r="AB64" t="n">
+        <v>1</v>
+      </c>
+      <c r="AC64" t="inlineStr">
+        <is>
+          <t>Taza rota</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>COM_X</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>COM</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>variante (regla de los 3 tiempos)</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>Pila de hojas de protocolo ordenada</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>pasado</t>
+        </is>
+      </c>
+      <c r="G65" t="n">
+        <v>1</v>
+      </c>
+      <c r="H65" t="n">
+        <v>2</v>
+      </c>
+      <c r="I65" t="n">
+        <v>0</v>
+      </c>
+      <c r="J65" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="X65" t="inlineStr">
+        <is>
+          <t>Solo visual: la misma cosa en otro tiempo</t>
+        </is>
+      </c>
+      <c r="Y65" t="n">
+        <v>7</v>
+      </c>
+      <c r="Z65" t="n">
+        <v>7</v>
+      </c>
+      <c r="AA65" t="n">
+        <v>2</v>
+      </c>
+      <c r="AB65" t="n">
+        <v>1</v>
+      </c>
+      <c r="AC65" t="inlineStr">
+        <is>
+          <t>Hojas de protocolo</t>
+        </is>
+      </c>
+      <c r="AF65" t="inlineStr">
+        <is>
+          <t>hoja_b</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>COM_Y</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>COM</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>variante (regla de los 3 tiempos)</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>Registro de transmisiones al día, sin la entrada 7.41</t>
+        </is>
+      </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>pasado</t>
+        </is>
+      </c>
+      <c r="G66" t="n">
+        <v>1</v>
+      </c>
+      <c r="H66" t="n">
+        <v>2</v>
+      </c>
+      <c r="I66" t="n">
+        <v>4</v>
+      </c>
+      <c r="J66" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="P66" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q66" t="inlineStr">
+        <is>
+          <t>T_COM_Y</t>
+        </is>
+      </c>
+      <c r="R66" t="n">
+        <v>4</v>
+      </c>
+      <c r="S66" t="inlineStr">
+        <is>
+          <t>A_COM_Y</t>
+        </is>
+      </c>
+      <c r="X66" t="inlineStr">
+        <is>
+          <t>Pista por comparación: en el presente (COM_H) la última entrada es 7.41</t>
+        </is>
+      </c>
+      <c r="Y66" t="n">
+        <v>6</v>
+      </c>
+      <c r="Z66" t="n">
+        <v>1</v>
+      </c>
+      <c r="AA66" t="n">
+        <v>2</v>
+      </c>
+      <c r="AB66" t="n">
+        <v>1</v>
+      </c>
+      <c r="AC66" t="inlineStr">
+        <is>
+          <t>Registro de transmisiones</t>
+        </is>
+      </c>
+      <c r="AF66" t="inlineStr">
+        <is>
+          <t>terminal_cian</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>COM_Z</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>COM</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>Z</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>variante (regla de los 3 tiempos)</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>Pantalla del registro apagada</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>futuro</t>
+        </is>
+      </c>
+      <c r="G67" t="n">
+        <v>1</v>
+      </c>
+      <c r="H67" t="n">
+        <v>2</v>
+      </c>
+      <c r="I67" t="n">
+        <v>0</v>
+      </c>
+      <c r="J67" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="X67" t="inlineStr">
+        <is>
+          <t>Solo visual: la misma cosa en otro tiempo</t>
+        </is>
+      </c>
+      <c r="Y67" t="n">
+        <v>6</v>
+      </c>
+      <c r="Z67" t="n">
+        <v>1</v>
+      </c>
+      <c r="AA67" t="n">
+        <v>2</v>
+      </c>
+      <c r="AB67" t="n">
+        <v>1</v>
+      </c>
+      <c r="AC67" t="inlineStr">
+        <is>
+          <t>Registro de transmisiones</t>
+        </is>
+      </c>
+      <c r="AF67" t="inlineStr">
+        <is>
+          <t>terminal_apagada</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>COM_AA</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>COM</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>AA</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>variante (regla de los 3 tiempos)</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>Plano de evacuación nuevo, plastificado</t>
+        </is>
+      </c>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>pasado</t>
+        </is>
+      </c>
+      <c r="G68" t="n">
+        <v>1</v>
+      </c>
+      <c r="H68" t="n">
         <v>3</v>
       </c>
-      <c r="AB62" t="n">
-        <v>1</v>
-      </c>
-      <c r="AC62" t="inlineStr">
-        <is>
-          <t>Destornillador</t>
+      <c r="I68" t="n">
+        <v>0</v>
+      </c>
+      <c r="J68" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="X68" t="inlineStr">
+        <is>
+          <t>Solo visual: la misma cosa en otro tiempo</t>
+        </is>
+      </c>
+      <c r="Y68" t="n">
+        <v>16</v>
+      </c>
+      <c r="Z68" t="n">
+        <v>8</v>
+      </c>
+      <c r="AA68" t="n">
+        <v>1</v>
+      </c>
+      <c r="AB68" t="n">
+        <v>2</v>
+      </c>
+      <c r="AC68" t="inlineStr">
+        <is>
+          <t>Plano de evacuación</t>
+        </is>
+      </c>
+      <c r="AF68" t="inlineStr">
+        <is>
+          <t>terminal_naranja</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>COM_AB</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>COM</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>AB</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>variante (regla de los 3 tiempos)</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>Lista de turnos descolorida</t>
+        </is>
+      </c>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>presente</t>
+        </is>
+      </c>
+      <c r="G69" t="n">
+        <v>1</v>
+      </c>
+      <c r="H69" t="n">
+        <v>3</v>
+      </c>
+      <c r="I69" t="n">
+        <v>0</v>
+      </c>
+      <c r="J69" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="X69" t="inlineStr">
+        <is>
+          <t>Solo visual: la misma cosa en otro tiempo</t>
+        </is>
+      </c>
+      <c r="Y69" t="n">
+        <v>16</v>
+      </c>
+      <c r="Z69" t="n">
+        <v>2</v>
+      </c>
+      <c r="AA69" t="n">
+        <v>1</v>
+      </c>
+      <c r="AB69" t="n">
+        <v>2</v>
+      </c>
+      <c r="AC69" t="inlineStr">
+        <is>
+          <t>Lista de turnos</t>
+        </is>
+      </c>
+      <c r="AF69" t="inlineStr">
+        <is>
+          <t>terminal_azul_b</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>COM_AC</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>COM</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>AC</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>variante (regla de los 3 tiempos)</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>Marca limpia en la pared donde estaba la lista de turnos</t>
+        </is>
+      </c>
+      <c r="F70" t="inlineStr">
+        <is>
+          <t>futuro</t>
+        </is>
+      </c>
+      <c r="G70" t="n">
+        <v>1</v>
+      </c>
+      <c r="H70" t="n">
+        <v>3</v>
+      </c>
+      <c r="I70" t="n">
+        <v>0</v>
+      </c>
+      <c r="J70" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="X70" t="inlineStr">
+        <is>
+          <t>Solo visual: la misma cosa en otro tiempo</t>
+        </is>
+      </c>
+      <c r="Y70" t="n">
+        <v>16</v>
+      </c>
+      <c r="Z70" t="n">
+        <v>2</v>
+      </c>
+      <c r="AA70" t="n">
+        <v>1</v>
+      </c>
+      <c r="AB70" t="n">
+        <v>2</v>
+      </c>
+      <c r="AC70" t="inlineStr">
+        <is>
+          <t>Pared</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>SCO_T</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>SCO</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>variante (regla de los 3 tiempos)</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>Silla en su lugar</t>
+        </is>
+      </c>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>pasado</t>
+        </is>
+      </c>
+      <c r="G71" t="n">
+        <v>1</v>
+      </c>
+      <c r="H71" t="n">
+        <v>1</v>
+      </c>
+      <c r="I71" t="n">
+        <v>0</v>
+      </c>
+      <c r="J71" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="X71" t="inlineStr">
+        <is>
+          <t>Solo visual: la misma cosa en otro tiempo</t>
+        </is>
+      </c>
+      <c r="Y71" t="n">
+        <v>2</v>
+      </c>
+      <c r="Z71" t="n">
+        <v>8</v>
+      </c>
+      <c r="AA71" t="n">
+        <v>1</v>
+      </c>
+      <c r="AB71" t="n">
+        <v>1</v>
+      </c>
+      <c r="AC71" t="inlineStr">
+        <is>
+          <t>Silla</t>
+        </is>
+      </c>
+      <c r="AF71" t="inlineStr">
+        <is>
+          <t>silla_frente</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>SCO_U</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>SCO</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>U</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>variante (regla de los 3 tiempos)</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>Mazo de cartas en su caja</t>
+        </is>
+      </c>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>pasado</t>
+        </is>
+      </c>
+      <c r="G72" t="n">
+        <v>1</v>
+      </c>
+      <c r="H72" t="n">
+        <v>1</v>
+      </c>
+      <c r="I72" t="n">
+        <v>0</v>
+      </c>
+      <c r="J72" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="X72" t="inlineStr">
+        <is>
+          <t>Solo visual: la misma cosa en otro tiempo</t>
+        </is>
+      </c>
+      <c r="Y72" t="n">
+        <v>12</v>
+      </c>
+      <c r="Z72" t="n">
+        <v>5</v>
+      </c>
+      <c r="AA72" t="n">
+        <v>2</v>
+      </c>
+      <c r="AB72" t="n">
+        <v>1</v>
+      </c>
+      <c r="AC72" t="inlineStr">
+        <is>
+          <t>Cartas</t>
+        </is>
+      </c>
+      <c r="AF72" t="inlineStr">
+        <is>
+          <t>caja_carton</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>SCO_V</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>SCO</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>variante (regla de los 3 tiempos)</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>Cartas desparramadas en el piso</t>
+        </is>
+      </c>
+      <c r="F73" t="inlineStr">
+        <is>
+          <t>futuro</t>
+        </is>
+      </c>
+      <c r="G73" t="n">
+        <v>1</v>
+      </c>
+      <c r="H73" t="n">
+        <v>1</v>
+      </c>
+      <c r="I73" t="n">
+        <v>0</v>
+      </c>
+      <c r="J73" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="X73" t="inlineStr">
+        <is>
+          <t>Solo visual: la misma cosa en otro tiempo</t>
+        </is>
+      </c>
+      <c r="Y73" t="n">
+        <v>12</v>
+      </c>
+      <c r="Z73" t="n">
+        <v>8</v>
+      </c>
+      <c r="AA73" t="n">
+        <v>2</v>
+      </c>
+      <c r="AB73" t="n">
+        <v>1</v>
+      </c>
+      <c r="AC73" t="inlineStr">
+        <is>
+          <t>Cartas</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>SCO_W</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>SCO</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>variante (regla de los 3 tiempos)</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>Pizarra de turnos en blanco, torcida</t>
+        </is>
+      </c>
+      <c r="F74" t="inlineStr">
+        <is>
+          <t>futuro</t>
+        </is>
+      </c>
+      <c r="G74" t="n">
+        <v>1</v>
+      </c>
+      <c r="H74" t="n">
+        <v>2</v>
+      </c>
+      <c r="I74" t="n">
+        <v>0</v>
+      </c>
+      <c r="J74" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="X74" t="inlineStr">
+        <is>
+          <t>Solo visual: la misma cosa en otro tiempo</t>
+        </is>
+      </c>
+      <c r="Y74" t="n">
+        <v>10</v>
+      </c>
+      <c r="Z74" t="n">
+        <v>1</v>
+      </c>
+      <c r="AA74" t="n">
+        <v>4</v>
+      </c>
+      <c r="AB74" t="n">
+        <v>1</v>
+      </c>
+      <c r="AC74" t="inlineStr">
+        <is>
+          <t>Pizarra de turnos</t>
+        </is>
+      </c>
+      <c r="AF74" t="inlineStr">
+        <is>
+          <t>panel_apagado</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>SCO_X</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>SCO</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>variante (regla de los 3 tiempos)</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>Dispensador de agua que gotea</t>
+        </is>
+      </c>
+      <c r="F75" t="inlineStr">
+        <is>
+          <t>presente</t>
+        </is>
+      </c>
+      <c r="G75" t="n">
+        <v>1</v>
+      </c>
+      <c r="H75" t="n">
+        <v>1</v>
+      </c>
+      <c r="I75" t="n">
+        <v>0</v>
+      </c>
+      <c r="J75" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="X75" t="inlineStr">
+        <is>
+          <t>Solo visual: la misma cosa en otro tiempo</t>
+        </is>
+      </c>
+      <c r="Y75" t="n">
+        <v>19</v>
+      </c>
+      <c r="Z75" t="n">
+        <v>1</v>
+      </c>
+      <c r="AA75" t="n">
+        <v>1</v>
+      </c>
+      <c r="AB75" t="n">
+        <v>2</v>
+      </c>
+      <c r="AC75" t="inlineStr">
+        <is>
+          <t>Dispensador de agua</t>
+        </is>
+      </c>
+      <c r="AF75" t="inlineStr">
+        <is>
+          <t>maquina_b</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>SCO_Y</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>SCO</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>variante (regla de los 3 tiempos)</t>
+        </is>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>Calendario tachado hasta el 112, descolorido</t>
+        </is>
+      </c>
+      <c r="F76" t="inlineStr">
+        <is>
+          <t>presente</t>
+        </is>
+      </c>
+      <c r="G76" t="n">
+        <v>1</v>
+      </c>
+      <c r="H76" t="n">
+        <v>2</v>
+      </c>
+      <c r="I76" t="n">
+        <v>0</v>
+      </c>
+      <c r="J76" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="X76" t="inlineStr">
+        <is>
+          <t>Solo visual: la misma cosa en otro tiempo</t>
+        </is>
+      </c>
+      <c r="Y76" t="n">
+        <v>5</v>
+      </c>
+      <c r="Z76" t="n">
+        <v>1</v>
+      </c>
+      <c r="AA76" t="n">
+        <v>2</v>
+      </c>
+      <c r="AB76" t="n">
+        <v>1</v>
+      </c>
+      <c r="AC76" t="inlineStr">
+        <is>
+          <t>Calendario</t>
+        </is>
+      </c>
+      <c r="AF76" t="inlineStr">
+        <is>
+          <t>hoja_c</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>SCO_Z</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>SCO</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>Z</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>variante (regla de los 3 tiempos)</t>
+        </is>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>Foto de la tripulación descolorida</t>
+        </is>
+      </c>
+      <c r="F77" t="inlineStr">
+        <is>
+          <t>presente</t>
+        </is>
+      </c>
+      <c r="G77" t="n">
+        <v>1</v>
+      </c>
+      <c r="H77" t="n">
+        <v>2</v>
+      </c>
+      <c r="I77" t="n">
+        <v>0</v>
+      </c>
+      <c r="J77" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="X77" t="inlineStr">
+        <is>
+          <t>Solo visual: la misma cosa en otro tiempo</t>
+        </is>
+      </c>
+      <c r="Y77" t="n">
+        <v>15</v>
+      </c>
+      <c r="Z77" t="n">
+        <v>1</v>
+      </c>
+      <c r="AA77" t="n">
+        <v>2</v>
+      </c>
+      <c r="AB77" t="n">
+        <v>1</v>
+      </c>
+      <c r="AC77" t="inlineStr">
+        <is>
+          <t>Foto de la tripulación</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>SCO_AA</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>SCO</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>AA</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>variante (regla de los 3 tiempos)</t>
+        </is>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>Marco de la foto con el vidrio roto</t>
+        </is>
+      </c>
+      <c r="F78" t="inlineStr">
+        <is>
+          <t>futuro</t>
+        </is>
+      </c>
+      <c r="G78" t="n">
+        <v>1</v>
+      </c>
+      <c r="H78" t="n">
+        <v>2</v>
+      </c>
+      <c r="I78" t="n">
+        <v>0</v>
+      </c>
+      <c r="J78" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="X78" t="inlineStr">
+        <is>
+          <t>Solo visual: la misma cosa en otro tiempo</t>
+        </is>
+      </c>
+      <c r="Y78" t="n">
+        <v>15</v>
+      </c>
+      <c r="Z78" t="n">
+        <v>1</v>
+      </c>
+      <c r="AA78" t="n">
+        <v>2</v>
+      </c>
+      <c r="AB78" t="n">
+        <v>1</v>
+      </c>
+      <c r="AC78" t="inlineStr">
+        <is>
+          <t>Marco roto</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>SCO_AB</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>SCO</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>AB</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>variante (regla de los 3 tiempos)</t>
+        </is>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>Reloj de pared andando</t>
+        </is>
+      </c>
+      <c r="F79" t="inlineStr">
+        <is>
+          <t>pasado</t>
+        </is>
+      </c>
+      <c r="G79" t="n">
+        <v>1</v>
+      </c>
+      <c r="H79" t="n">
+        <v>2</v>
+      </c>
+      <c r="I79" t="n">
+        <v>0</v>
+      </c>
+      <c r="J79" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="X79" t="inlineStr">
+        <is>
+          <t>Solo visual: la misma cosa en otro tiempo</t>
+        </is>
+      </c>
+      <c r="Y79" t="n">
+        <v>18</v>
+      </c>
+      <c r="Z79" t="n">
+        <v>1</v>
+      </c>
+      <c r="AA79" t="n">
+        <v>1</v>
+      </c>
+      <c r="AB79" t="n">
+        <v>1</v>
+      </c>
+      <c r="AC79" t="inlineStr">
+        <is>
+          <t>Reloj de pared</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>SCO_AC</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>SCO</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>AC</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>variante (regla de los 3 tiempos)</t>
+        </is>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>Reloj caído en el piso, sin agujas</t>
+        </is>
+      </c>
+      <c r="F80" t="inlineStr">
+        <is>
+          <t>futuro</t>
+        </is>
+      </c>
+      <c r="G80" t="n">
+        <v>1</v>
+      </c>
+      <c r="H80" t="n">
+        <v>2</v>
+      </c>
+      <c r="I80" t="n">
+        <v>0</v>
+      </c>
+      <c r="J80" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="X80" t="inlineStr">
+        <is>
+          <t>Solo visual: la misma cosa en otro tiempo</t>
+        </is>
+      </c>
+      <c r="Y80" t="n">
+        <v>18</v>
+      </c>
+      <c r="Z80" t="n">
+        <v>2</v>
+      </c>
+      <c r="AA80" t="n">
+        <v>1</v>
+      </c>
+      <c r="AB80" t="n">
+        <v>1</v>
+      </c>
+      <c r="AC80" t="inlineStr">
+        <is>
+          <t>Reloj caído</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>SCO_AD</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>SCO</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>AD</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>variante (regla de los 3 tiempos)</t>
+        </is>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>Chaqueta colgada en la pared</t>
+        </is>
+      </c>
+      <c r="F81" t="inlineStr">
+        <is>
+          <t>pasado</t>
+        </is>
+      </c>
+      <c r="G81" t="n">
+        <v>1</v>
+      </c>
+      <c r="H81" t="n">
+        <v>2</v>
+      </c>
+      <c r="I81" t="n">
+        <v>0</v>
+      </c>
+      <c r="J81" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="X81" t="inlineStr">
+        <is>
+          <t>Solo visual: la misma cosa en otro tiempo</t>
+        </is>
+      </c>
+      <c r="Y81" t="n">
+        <v>17</v>
+      </c>
+      <c r="Z81" t="n">
+        <v>1</v>
+      </c>
+      <c r="AA81" t="n">
+        <v>1</v>
+      </c>
+      <c r="AB81" t="n">
+        <v>1</v>
+      </c>
+      <c r="AC81" t="inlineStr">
+        <is>
+          <t>Chaqueta</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>SCO_AE</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>SCO</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>AE</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>variante (regla de los 3 tiempos)</t>
+        </is>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>Chaqueta en el piso, gastada</t>
+        </is>
+      </c>
+      <c r="F82" t="inlineStr">
+        <is>
+          <t>futuro</t>
+        </is>
+      </c>
+      <c r="G82" t="n">
+        <v>1</v>
+      </c>
+      <c r="H82" t="n">
+        <v>2</v>
+      </c>
+      <c r="I82" t="n">
+        <v>0</v>
+      </c>
+      <c r="J82" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="X82" t="inlineStr">
+        <is>
+          <t>Solo visual: la misma cosa en otro tiempo</t>
+        </is>
+      </c>
+      <c r="Y82" t="n">
+        <v>16</v>
+      </c>
+      <c r="Z82" t="n">
+        <v>8</v>
+      </c>
+      <c r="AA82" t="n">
+        <v>1</v>
+      </c>
+      <c r="AB82" t="n">
+        <v>1</v>
+      </c>
+      <c r="AC82" t="inlineStr">
+        <is>
+          <t>Chaqueta</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>PTA_F</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>PTA</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>variante (regla de los 3 tiempos)</t>
+        </is>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>Soporte con la placa tapada por el plástico protector (no se lee)</t>
+        </is>
+      </c>
+      <c r="F83" t="inlineStr">
+        <is>
+          <t>pasado</t>
+        </is>
+      </c>
+      <c r="G83" t="n">
+        <v>1</v>
+      </c>
+      <c r="H83" t="n">
+        <v>2</v>
+      </c>
+      <c r="I83" t="n">
+        <v>0</v>
+      </c>
+      <c r="J83" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="X83" t="inlineStr">
+        <is>
+          <t>Solo visual: la misma cosa en otro tiempo</t>
+        </is>
+      </c>
+      <c r="Y83" t="n">
+        <v>6</v>
+      </c>
+      <c r="Z83" t="n">
+        <v>1</v>
+      </c>
+      <c r="AA83" t="n">
+        <v>1</v>
+      </c>
+      <c r="AB83" t="n">
+        <v>1</v>
+      </c>
+      <c r="AC83" t="inlineStr">
+        <is>
+          <t>Soporte de placa</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>PTA_G</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>PTA</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>variante (regla de los 3 tiempos)</t>
+        </is>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>Soporte de placa oxidado, vacío</t>
+        </is>
+      </c>
+      <c r="F84" t="inlineStr">
+        <is>
+          <t>futuro</t>
+        </is>
+      </c>
+      <c r="G84" t="n">
+        <v>1</v>
+      </c>
+      <c r="H84" t="n">
+        <v>2</v>
+      </c>
+      <c r="I84" t="n">
+        <v>0</v>
+      </c>
+      <c r="J84" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="X84" t="inlineStr">
+        <is>
+          <t>Solo visual: la misma cosa en otro tiempo</t>
+        </is>
+      </c>
+      <c r="Y84" t="n">
+        <v>6</v>
+      </c>
+      <c r="Z84" t="n">
+        <v>1</v>
+      </c>
+      <c r="AA84" t="n">
+        <v>1</v>
+      </c>
+      <c r="AB84" t="n">
+        <v>1</v>
+      </c>
+      <c r="AC84" t="inlineStr">
+        <is>
+          <t>Soporte de placa</t>
         </is>
       </c>
     </row>
@@ -7450,7 +10331,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I18"/>
+  <dimension ref="A1:K18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -7510,6 +10391,16 @@
           <t>en_futuro</t>
         </is>
       </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>sprite</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>sprite_futuro</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -7544,6 +10435,11 @@
           <t>sí</t>
         </is>
       </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>consola_larga</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -7583,6 +10479,11 @@
           <t>roto</t>
         </is>
       </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>mesa_azul repetir</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -7617,6 +10518,11 @@
           <t>sí</t>
         </is>
       </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>estantes</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -7651,6 +10557,11 @@
           <t>sí</t>
         </is>
       </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>mesa_oscura repetir</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -7685,6 +10596,11 @@
           <t>sí</t>
         </is>
       </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>cajitas</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -7724,6 +10640,11 @@
           <t>roto</t>
         </is>
       </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>mesa_naranja repetir</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -7758,6 +10679,11 @@
           <t>caído</t>
         </is>
       </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>silla_frente</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -7792,6 +10718,11 @@
           <t>caído</t>
         </is>
       </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>silla_frente</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -7826,6 +10757,11 @@
           <t>caído</t>
         </is>
       </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>silla_frente</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -7860,6 +10796,11 @@
           <t>caído</t>
         </is>
       </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>silla_espalda</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -7894,6 +10835,11 @@
           <t>caído</t>
         </is>
       </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>silla_espalda</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -7928,6 +10874,11 @@
           <t>caído</t>
         </is>
       </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>silla_espalda</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -7962,6 +10913,11 @@
           <t>caído</t>
         </is>
       </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>silla_espalda</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -7996,6 +10952,11 @@
           <t>caído</t>
         </is>
       </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>silla_lado</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -8030,6 +10991,11 @@
           <t>sí</t>
         </is>
       </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>estante_colgado</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -8059,6 +11025,11 @@
           <t>sí</t>
         </is>
       </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>ninguno</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -8086,6 +11057,11 @@
       <c r="H18" t="inlineStr">
         <is>
           <t>sí</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>ninguno</t>
         </is>
       </c>
     </row>
@@ -8100,7 +11076,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D133"/>
+  <dimension ref="A1:D135"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -10768,6 +13744,46 @@
       <c r="D133" t="inlineStr">
         <is>
           <t>¿En qué puedo ayudarle?</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>T_COM_Y</t>
+        </is>
+      </c>
+      <c r="B134" t="n">
+        <v>1</v>
+      </c>
+      <c r="C134" t="inlineStr">
+        <is>
+          <t>PERSONAJE</t>
+        </is>
+      </c>
+      <c r="D134" t="inlineStr">
+        <is>
+          <t>Registro de transmisiones. Todo rutinario.</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>T_COM_Y</t>
+        </is>
+      </c>
+      <c r="B135" t="n">
+        <v>2</v>
+      </c>
+      <c r="C135" t="inlineStr">
+        <is>
+          <t>PERSONAJE</t>
+        </is>
+      </c>
+      <c r="D135" t="inlineStr">
+        <is>
+          <t>La última entrada es de un control de rutina. No hay nada en 7.41.</t>
         </is>
       </c>
     </row>
@@ -10783,7 +13799,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B26"/>
+  <dimension ref="A1:B27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -11099,6 +14115,18 @@
       <c r="B26" t="inlineStr">
         <is>
           <t>Encontré un destornillador para abrir el panel. Me falta una pinza para el cable.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>A_COM_Y</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Vi el registro de transmisiones sin ninguna entrada en 7.41.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Sala común: salida trabada a la derecha
</commit_message>
<xml_diff>
--- a/planilla/contenido_alfa.xlsx
+++ b/planilla/contenido_alfa.xlsx
@@ -6833,7 +6833,7 @@
       </c>
       <c r="E50" s="2" t="inlineStr">
         <is>
-          <t>Puertas hacia el resto de la nave, trabadas</t>
+          <t>Puertas hacia el resto de la nave (salida de la derecha), trabadas</t>
         </is>
       </c>
       <c r="F50" s="2" t="inlineStr">
@@ -6876,14 +6876,14 @@
       <c r="W50" s="2" t="n"/>
       <c r="X50" s="2" t="inlineStr">
         <is>
-          <t>Confirmado en el paso 9</t>
+          <t>Al lado del recoveco de la derecha; la puerta la dibuja la nave (sala.salida_trabada_derecha)</t>
         </is>
       </c>
       <c r="Y50" s="3" t="n">
         <v>21</v>
       </c>
       <c r="Z50" s="3" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="AA50" s="3" t="n">
         <v>1</v>
@@ -6894,6 +6894,11 @@
       <c r="AC50" s="3" t="inlineStr">
         <is>
           <t>Puertas hacia el resto de la nave</t>
+        </is>
+      </c>
+      <c r="AF50" t="inlineStr">
+        <is>
+          <t>ninguno</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Arte al doble y salas a la mitad de tiles
</commit_message>
<xml_diff>
--- a/planilla/contenido_alfa.xlsx
+++ b/planilla/contenido_alfa.xlsx
@@ -458,7 +458,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A36"/>
+  <dimension ref="A1:A37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="140" customWidth="1" min="1" max="1"/>
@@ -698,6 +698,13 @@
       <c r="A36" t="inlineStr">
         <is>
           <t>sprite vacío = cuadro de color (greybox, cuando no hay sprite: taza, pinza, foto…). 'ninguno' = no se dibuja (lo muestra el mueble de abajo). sprite_usado = cómo se ve después de usarlo (la silla levantada, el panel arreglado).</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Escala x2 (22/10/2026): el arte se dibuja al doble (Medidas.ARTE = 2, tile de 96 en el mundo). Las salas pasaron a la mitad de tiles (mando 10x6, comunicaciones 10x6, sala común 12x6, sala de la puerta 6x4) y todo se reubicó. Las filas 4-5 de mando, comunicaciones y la sala común se dejan libres: ahí están las aberturas de los pasillos de costado.</t>
         </is>
       </c>
     </row>
@@ -2359,13 +2366,13 @@
         </is>
       </c>
       <c r="Y2" s="3" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="Z2" s="3" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="AA2" s="3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AB2" s="3" t="n">
         <v>1</v>
@@ -2447,13 +2454,13 @@
       <c r="W3" s="2" t="n"/>
       <c r="X3" s="2" t="inlineStr"/>
       <c r="Y3" s="3" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="Z3" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="AA3" s="3" t="n">
         <v>2</v>
-      </c>
-      <c r="AA3" s="3" t="n">
-        <v>4</v>
       </c>
       <c r="AB3" s="3" t="n">
         <v>1</v>
@@ -2547,13 +2554,13 @@
         </is>
       </c>
       <c r="Y4" s="3" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="Z4" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="AA4" s="3" t="n">
         <v>2</v>
-      </c>
-      <c r="AA4" s="3" t="n">
-        <v>4</v>
       </c>
       <c r="AB4" s="3" t="n">
         <v>1</v>
@@ -2647,13 +2654,13 @@
         </is>
       </c>
       <c r="Y5" s="3" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="Z5" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="AA5" s="3" t="n">
         <v>2</v>
-      </c>
-      <c r="AA5" s="3" t="n">
-        <v>4</v>
       </c>
       <c r="AB5" s="3" t="n">
         <v>1</v>
@@ -2747,13 +2754,13 @@
         </is>
       </c>
       <c r="Y6" s="3" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="Z6" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="AA6" s="3" t="n">
         <v>2</v>
-      </c>
-      <c r="AA6" s="3" t="n">
-        <v>4</v>
       </c>
       <c r="AB6" s="3" t="n">
         <v>1</v>
@@ -2843,13 +2850,13 @@
       <c r="W7" s="2" t="n"/>
       <c r="X7" s="2" t="inlineStr"/>
       <c r="Y7" s="3" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="Z7" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="AA7" s="3" t="n">
         <v>2</v>
-      </c>
-      <c r="AA7" s="3" t="n">
-        <v>4</v>
       </c>
       <c r="AB7" s="3" t="n">
         <v>1</v>
@@ -2939,13 +2946,13 @@
       <c r="W8" s="2" t="n"/>
       <c r="X8" s="2" t="inlineStr"/>
       <c r="Y8" s="3" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="Z8" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="AA8" s="3" t="n">
         <v>2</v>
-      </c>
-      <c r="AA8" s="3" t="n">
-        <v>4</v>
       </c>
       <c r="AB8" s="3" t="n">
         <v>1</v>
@@ -3035,13 +3042,13 @@
       <c r="W9" s="2" t="n"/>
       <c r="X9" s="2" t="inlineStr"/>
       <c r="Y9" s="3" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="Z9" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="AA9" s="3" t="n">
         <v>2</v>
-      </c>
-      <c r="AA9" s="3" t="n">
-        <v>4</v>
       </c>
       <c r="AB9" s="3" t="n">
         <v>1</v>
@@ -3131,13 +3138,13 @@
       <c r="W10" s="2" t="n"/>
       <c r="X10" s="2" t="inlineStr"/>
       <c r="Y10" s="3" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="Z10" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="AA10" s="3" t="n">
         <v>2</v>
-      </c>
-      <c r="AA10" s="3" t="n">
-        <v>4</v>
       </c>
       <c r="AB10" s="3" t="n">
         <v>1</v>
@@ -3235,13 +3242,13 @@
         </is>
       </c>
       <c r="Y11" s="3" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="Z11" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="AA11" s="3" t="n">
         <v>2</v>
-      </c>
-      <c r="AA11" s="3" t="n">
-        <v>4</v>
       </c>
       <c r="AB11" s="3" t="n">
         <v>1</v>
@@ -3323,13 +3330,13 @@
       <c r="W12" s="2" t="n"/>
       <c r="X12" s="2" t="inlineStr"/>
       <c r="Y12" s="3" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="Z12" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="AA12" s="3" t="n">
         <v>2</v>
-      </c>
-      <c r="AA12" s="3" t="n">
-        <v>4</v>
       </c>
       <c r="AB12" s="3" t="n">
         <v>1</v>
@@ -3419,13 +3426,13 @@
       <c r="W13" s="2" t="n"/>
       <c r="X13" s="2" t="n"/>
       <c r="Y13" s="3" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="Z13" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="AA13" s="3" t="n">
         <v>2</v>
-      </c>
-      <c r="AA13" s="3" t="n">
-        <v>4</v>
       </c>
       <c r="AB13" s="3" t="n">
         <v>1</v>
@@ -3515,13 +3522,13 @@
       <c r="W14" s="2" t="n"/>
       <c r="X14" s="2" t="inlineStr"/>
       <c r="Y14" s="3" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="Z14" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="AA14" s="3" t="n">
         <v>2</v>
-      </c>
-      <c r="AA14" s="3" t="n">
-        <v>4</v>
       </c>
       <c r="AB14" s="3" t="n">
         <v>1</v>
@@ -3603,10 +3610,10 @@
       <c r="W15" s="2" t="n"/>
       <c r="X15" s="2" t="inlineStr"/>
       <c r="Y15" s="3" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="Z15" s="3" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="AA15" s="3" t="n">
         <v>1</v>
@@ -3692,13 +3699,13 @@
       <c r="W16" s="2" t="n"/>
       <c r="X16" s="2" t="inlineStr"/>
       <c r="Y16" s="3" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="Z16" s="3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AA16" s="3" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="AB16" s="3" t="n">
         <v>1</v>
@@ -3786,10 +3793,10 @@
       <c r="W17" s="2" t="n"/>
       <c r="X17" s="2" t="inlineStr"/>
       <c r="Y17" s="3" t="n">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="Z17" s="3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AA17" s="3" t="n">
         <v>3</v>
@@ -3880,10 +3887,10 @@
       <c r="W18" s="2" t="n"/>
       <c r="X18" s="2" t="inlineStr"/>
       <c r="Y18" s="3" t="n">
-        <v>16</v>
+        <v>9</v>
       </c>
       <c r="Z18" s="3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AA18" s="3" t="n">
         <v>1</v>
@@ -3980,13 +3987,13 @@
       <c r="W19" s="2" t="n"/>
       <c r="X19" s="2" t="inlineStr"/>
       <c r="Y19" s="3" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="Z19" s="3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AA19" s="3" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="AB19" s="3" t="n">
         <v>1</v>
@@ -4074,10 +4081,10 @@
       <c r="W20" s="2" t="n"/>
       <c r="X20" s="2" t="inlineStr"/>
       <c r="Y20" s="3" t="n">
-        <v>16</v>
+        <v>0</v>
       </c>
       <c r="Z20" s="3" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="AA20" s="3" t="n">
         <v>1</v>
@@ -4162,13 +4169,13 @@
       <c r="W21" s="2" t="n"/>
       <c r="X21" s="2" t="inlineStr"/>
       <c r="Y21" s="3" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="Z21" s="3" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="AA21" s="3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AB21" s="3" t="n">
         <v>1</v>
@@ -4256,13 +4263,13 @@
       <c r="W22" s="2" t="n"/>
       <c r="X22" s="2" t="inlineStr"/>
       <c r="Y22" s="3" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="Z22" s="3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AA22" s="3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AB22" s="3" t="n">
         <v>1</v>
@@ -4350,13 +4357,13 @@
       <c r="W23" s="2" t="n"/>
       <c r="X23" s="2" t="inlineStr"/>
       <c r="Y23" s="3" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="Z23" s="3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AA23" s="3" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="AB23" s="3" t="n">
         <v>1</v>
@@ -4442,10 +4449,10 @@
         </is>
       </c>
       <c r="Y24" s="3" t="n">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="Z24" s="3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AA24" s="3" t="n">
         <v>3</v>
@@ -4530,10 +4537,10 @@
       <c r="W25" s="2" t="n"/>
       <c r="X25" s="2" t="inlineStr"/>
       <c r="Y25" s="3" t="n">
-        <v>16</v>
+        <v>0</v>
       </c>
       <c r="Z25" s="3" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="AA25" s="3" t="n">
         <v>1</v>
@@ -4636,10 +4643,10 @@
       <c r="W26" s="2" t="n"/>
       <c r="X26" s="2" t="inlineStr"/>
       <c r="Y26" s="3" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="Z26" s="3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AA26" s="3" t="n">
         <v>1</v>
@@ -4748,10 +4755,10 @@
         </is>
       </c>
       <c r="Y27" s="3" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="Z27" s="3" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="AA27" s="3" t="n">
         <v>1</v>
@@ -4837,10 +4844,10 @@
         </is>
       </c>
       <c r="Y28" s="3" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="Z28" s="3" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="AA28" s="3" t="n">
         <v>1</v>
@@ -4942,10 +4949,10 @@
         </is>
       </c>
       <c r="Y29" s="3" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="Z29" s="3" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="AA29" s="3" t="n">
         <v>1</v>
@@ -5031,10 +5038,10 @@
         </is>
       </c>
       <c r="Y30" s="3" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="Z30" s="3" t="n">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="AA30" s="3" t="n">
         <v>1</v>
@@ -5129,10 +5136,10 @@
         </is>
       </c>
       <c r="Y31" s="3" t="n">
-        <v>17</v>
+        <v>9</v>
       </c>
       <c r="Z31" s="3" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="AA31" s="3" t="n">
         <v>1</v>
@@ -5223,16 +5230,16 @@
       <c r="W32" s="2" t="n"/>
       <c r="X32" s="2" t="inlineStr"/>
       <c r="Y32" s="3" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="Z32" s="3" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="AA32" s="3" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="AB32" s="3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AC32" s="3" t="inlineStr">
         <is>
@@ -5311,16 +5318,16 @@
       <c r="W33" s="2" t="n"/>
       <c r="X33" s="2" t="inlineStr"/>
       <c r="Y33" s="3" t="n">
-        <v>19</v>
+        <v>11</v>
       </c>
       <c r="Z33" s="3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AA33" s="3" t="n">
         <v>1</v>
       </c>
       <c r="AB33" s="3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AC33" s="3" t="inlineStr">
         <is>
@@ -5405,16 +5412,16 @@
       <c r="W34" s="2" t="n"/>
       <c r="X34" s="2" t="inlineStr"/>
       <c r="Y34" s="3" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="Z34" s="3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AA34" s="3" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="AB34" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AC34" s="3" t="inlineStr">
         <is>
@@ -5503,10 +5510,10 @@
         </is>
       </c>
       <c r="Y35" s="3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="Z35" s="3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AA35" s="3" t="n">
         <v>1</v>
@@ -5596,13 +5603,13 @@
         </is>
       </c>
       <c r="Y36" s="3" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="Z36" s="3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AA36" s="3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AB36" s="3" t="n">
         <v>1</v>
@@ -5688,13 +5695,13 @@
         </is>
       </c>
       <c r="Y37" s="3" t="n">
-        <v>15</v>
+        <v>8</v>
       </c>
       <c r="Z37" s="3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AA37" s="3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AB37" s="3" t="n">
         <v>1</v>
@@ -5777,13 +5784,13 @@
       <c r="W38" s="2" t="n"/>
       <c r="X38" s="2" t="inlineStr"/>
       <c r="Y38" s="3" t="n">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="Z38" s="3" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="AA38" s="3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AB38" s="3" t="n">
         <v>1</v>
@@ -5866,10 +5873,10 @@
       <c r="W39" s="2" t="n"/>
       <c r="X39" s="2" t="inlineStr"/>
       <c r="Y39" s="3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="Z39" s="3" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="AA39" s="3" t="n">
         <v>1</v>
@@ -5959,10 +5966,10 @@
       <c r="W40" s="2" t="n"/>
       <c r="X40" s="2" t="inlineStr"/>
       <c r="Y40" s="3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="Z40" s="3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AA40" s="3" t="n">
         <v>1</v>
@@ -6056,10 +6063,10 @@
       <c r="W41" s="2" t="n"/>
       <c r="X41" s="2" t="inlineStr"/>
       <c r="Y41" s="3" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="Z41" s="3" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="AA41" s="3" t="n">
         <v>1</v>
@@ -6145,16 +6152,16 @@
       <c r="W42" s="2" t="n"/>
       <c r="X42" s="2" t="inlineStr"/>
       <c r="Y42" s="3" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="Z42" s="3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AA42" s="3" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="AB42" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AC42" s="3" t="inlineStr">
         <is>
@@ -6243,10 +6250,10 @@
         </is>
       </c>
       <c r="Y43" s="3" t="n">
-        <v>18</v>
+        <v>10</v>
       </c>
       <c r="Z43" s="3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AA43" s="3" t="n">
         <v>1</v>
@@ -6330,10 +6337,10 @@
         </is>
       </c>
       <c r="Y44" s="3" t="n">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="Z44" s="3" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="AA44" s="3" t="n">
         <v>1</v>
@@ -6413,16 +6420,16 @@
       <c r="W45" s="2" t="n"/>
       <c r="X45" s="2" t="inlineStr"/>
       <c r="Y45" s="3" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="Z45" s="3" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="AA45" s="3" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="AB45" s="3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AC45" s="3" t="inlineStr">
         <is>
@@ -6515,10 +6522,10 @@
       <c r="W46" s="2" t="n"/>
       <c r="X46" s="2" t="inlineStr"/>
       <c r="Y46" s="3" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="Z46" s="3" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="AA46" s="3" t="n">
         <v>1</v>
@@ -6602,13 +6609,13 @@
         </is>
       </c>
       <c r="Y47" s="3" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="Z47" s="3" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="AA47" s="3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AB47" s="3" t="n">
         <v>1</v>
@@ -6694,16 +6701,16 @@
         </is>
       </c>
       <c r="Y48" s="3" t="n">
-        <v>19</v>
+        <v>11</v>
       </c>
       <c r="Z48" s="3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AA48" s="3" t="n">
         <v>1</v>
       </c>
       <c r="AB48" s="3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AC48" s="3" t="inlineStr">
         <is>
@@ -6788,10 +6795,10 @@
         </is>
       </c>
       <c r="Y49" s="3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="Z49" s="3" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="AA49" s="3" t="n">
         <v>1</v>
@@ -6880,10 +6887,10 @@
         </is>
       </c>
       <c r="Y50" s="3" t="n">
-        <v>21</v>
+        <v>11</v>
       </c>
       <c r="Z50" s="3" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="AA50" s="3" t="n">
         <v>1</v>
@@ -6974,7 +6981,7 @@
       <c r="W51" s="2" t="n"/>
       <c r="X51" s="2" t="inlineStr"/>
       <c r="Y51" s="3" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="Z51" s="3" t="n">
         <v>0</v>
@@ -7062,10 +7069,10 @@
       <c r="W52" s="2" t="n"/>
       <c r="X52" s="2" t="inlineStr"/>
       <c r="Y52" s="3" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="Z52" s="3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AA52" s="3" t="n">
         <v>1</v>
@@ -7151,7 +7158,7 @@
       <c r="W53" s="2" t="n"/>
       <c r="X53" s="2" t="inlineStr"/>
       <c r="Y53" s="3" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="Z53" s="3" t="n">
         <v>0</v>
@@ -7239,7 +7246,7 @@
       <c r="W54" s="2" t="n"/>
       <c r="X54" s="2" t="inlineStr"/>
       <c r="Y54" s="3" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="Z54" s="3" t="n">
         <v>0</v>
@@ -7327,7 +7334,7 @@
       <c r="W55" s="2" t="n"/>
       <c r="X55" s="2" t="inlineStr"/>
       <c r="Y55" s="3" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="Z55" s="3" t="n">
         <v>1</v>
@@ -7414,10 +7421,10 @@
         </is>
       </c>
       <c r="Y56" s="3" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="Z56" s="3" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="AA56" s="3" t="n">
         <v>1</v>
@@ -7523,10 +7530,10 @@
         </is>
       </c>
       <c r="Y57" s="3" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="Z57" s="3" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="AA57" s="3" t="n">
         <v>1</v>
@@ -7614,13 +7621,13 @@
         </is>
       </c>
       <c r="Y58" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="Z58" t="n">
+        <v>1</v>
+      </c>
+      <c r="AA58" t="n">
         <v>2</v>
-      </c>
-      <c r="AA58" t="n">
-        <v>4</v>
       </c>
       <c r="AB58" t="n">
         <v>1</v>
@@ -7695,13 +7702,13 @@
         </is>
       </c>
       <c r="Y59" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="Z59" t="n">
+        <v>1</v>
+      </c>
+      <c r="AA59" t="n">
         <v>2</v>
-      </c>
-      <c r="AA59" t="n">
-        <v>4</v>
       </c>
       <c r="AB59" t="n">
         <v>1</v>
@@ -7813,10 +7820,10 @@
         </is>
       </c>
       <c r="Y60" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="Z60" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="AA60" t="n">
         <v>1</v>
@@ -7925,13 +7932,13 @@
         </is>
       </c>
       <c r="Y61" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="Z61" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="AA61" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AB61" t="n">
         <v>1</v>
@@ -8045,10 +8052,10 @@
         </is>
       </c>
       <c r="Y62" t="n">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="Z62" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AA62" t="n">
         <v>1</v>
@@ -8113,10 +8120,10 @@
         </is>
       </c>
       <c r="Y63" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="Z63" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="AA63" t="n">
         <v>1</v>
@@ -8181,10 +8188,10 @@
         </is>
       </c>
       <c r="Y64" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="Z64" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="AA64" t="n">
         <v>1</v>
@@ -8249,13 +8256,13 @@
         </is>
       </c>
       <c r="Y65" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="Z65" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="AA65" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AB65" t="n">
         <v>1</v>
@@ -8338,13 +8345,13 @@
         </is>
       </c>
       <c r="Y66" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="Z66" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AA66" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AB66" t="n">
         <v>1</v>
@@ -8411,13 +8418,13 @@
         </is>
       </c>
       <c r="Y67" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="Z67" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AA67" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AB67" t="n">
         <v>1</v>
@@ -8484,10 +8491,10 @@
         </is>
       </c>
       <c r="Y68" t="n">
-        <v>16</v>
+        <v>0</v>
       </c>
       <c r="Z68" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="AA68" t="n">
         <v>1</v>
@@ -8557,10 +8564,10 @@
         </is>
       </c>
       <c r="Y69" t="n">
-        <v>16</v>
+        <v>9</v>
       </c>
       <c r="Z69" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AA69" t="n">
         <v>1</v>
@@ -8630,10 +8637,10 @@
         </is>
       </c>
       <c r="Y70" t="n">
-        <v>16</v>
+        <v>9</v>
       </c>
       <c r="Z70" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AA70" t="n">
         <v>1</v>
@@ -8698,10 +8705,10 @@
         </is>
       </c>
       <c r="Y71" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="Z71" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="AA71" t="n">
         <v>1</v>
@@ -8771,13 +8778,13 @@
         </is>
       </c>
       <c r="Y72" t="n">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="Z72" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="AA72" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AB72" t="n">
         <v>1</v>
@@ -8844,13 +8851,13 @@
         </is>
       </c>
       <c r="Y73" t="n">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="Z73" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="AA73" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AB73" t="n">
         <v>1</v>
@@ -8912,16 +8919,16 @@
         </is>
       </c>
       <c r="Y74" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="Z74" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AA74" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="AB74" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AC74" t="inlineStr">
         <is>
@@ -8985,16 +8992,16 @@
         </is>
       </c>
       <c r="Y75" t="n">
-        <v>19</v>
+        <v>11</v>
       </c>
       <c r="Z75" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AA75" t="n">
         <v>1</v>
       </c>
       <c r="AB75" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AC75" t="inlineStr">
         <is>
@@ -9058,13 +9065,13 @@
         </is>
       </c>
       <c r="Y76" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="Z76" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AA76" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AB76" t="n">
         <v>1</v>
@@ -9131,13 +9138,13 @@
         </is>
       </c>
       <c r="Y77" t="n">
-        <v>15</v>
+        <v>8</v>
       </c>
       <c r="Z77" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AA77" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AB77" t="n">
         <v>1</v>
@@ -9199,13 +9206,13 @@
         </is>
       </c>
       <c r="Y78" t="n">
-        <v>15</v>
+        <v>8</v>
       </c>
       <c r="Z78" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AA78" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AB78" t="n">
         <v>1</v>
@@ -9267,10 +9274,10 @@
         </is>
       </c>
       <c r="Y79" t="n">
-        <v>18</v>
+        <v>10</v>
       </c>
       <c r="Z79" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AA79" t="n">
         <v>1</v>
@@ -9335,10 +9342,10 @@
         </is>
       </c>
       <c r="Y80" t="n">
-        <v>18</v>
+        <v>10</v>
       </c>
       <c r="Z80" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AA80" t="n">
         <v>1</v>
@@ -9403,10 +9410,10 @@
         </is>
       </c>
       <c r="Y81" t="n">
-        <v>17</v>
+        <v>9</v>
       </c>
       <c r="Z81" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AA81" t="n">
         <v>1</v>
@@ -9471,10 +9478,10 @@
         </is>
       </c>
       <c r="Y82" t="n">
-        <v>16</v>
+        <v>9</v>
       </c>
       <c r="Z82" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="AA82" t="n">
         <v>1</v>
@@ -9539,10 +9546,10 @@
         </is>
       </c>
       <c r="Y83" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="Z83" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AA83" t="n">
         <v>1</v>
@@ -9607,10 +9614,10 @@
         </is>
       </c>
       <c r="Y84" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="Z84" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AA84" t="n">
         <v>1</v>
@@ -10419,16 +10426,16 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="D2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E2" t="n">
         <v>6</v>
       </c>
       <c r="F2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
@@ -10458,13 +10465,13 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E3" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="F3" t="n">
         <v>1</v>
@@ -10502,10 +10509,10 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="D4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E4" t="n">
         <v>3</v>
@@ -10541,16 +10548,16 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="D5" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="E5" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="F5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
@@ -10580,13 +10587,13 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="D6" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="E6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F6" t="n">
         <v>1</v>
@@ -10619,16 +10626,16 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="D7" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="E7" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="F7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
@@ -10663,10 +10670,10 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="D8" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="E8" t="n">
         <v>1</v>
@@ -10702,10 +10709,10 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="D9" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="E9" t="n">
         <v>1</v>
@@ -10741,10 +10748,10 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>14</v>
+        <v>3</v>
       </c>
       <c r="D10" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E10" t="n">
         <v>1</v>
@@ -10764,7 +10771,7 @@
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>silla_frente</t>
+          <t>silla_espalda</t>
         </is>
       </c>
     </row>
@@ -10780,10 +10787,10 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="D11" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="E11" t="n">
         <v>1</v>
@@ -10819,10 +10826,10 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="D12" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="E12" t="n">
         <v>1</v>
@@ -10858,10 +10865,10 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="D13" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="E13" t="n">
         <v>1</v>
@@ -10897,10 +10904,10 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>14</v>
+        <v>2</v>
       </c>
       <c r="D14" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="E14" t="n">
         <v>1</v>
@@ -10920,7 +10927,7 @@
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>silla_espalda</t>
+          <t>silla_lado espejo</t>
         </is>
       </c>
     </row>
@@ -10936,10 +10943,10 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>15</v>
+        <v>9</v>
       </c>
       <c r="D15" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="E15" t="n">
         <v>1</v>
@@ -10975,10 +10982,10 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D16" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E16" t="n">
         <v>3</v>
@@ -11014,13 +11021,13 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="D17" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E17" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F17" t="n">
         <v>1</v>
@@ -11048,16 +11055,16 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>19</v>
+        <v>11</v>
       </c>
       <c r="D18" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E18" t="n">
         <v>1</v>
       </c>
       <c r="F18" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H18" t="inlineStr">
         <is>

</xml_diff>